<commit_message>
Sparkling Daily — full planning tool (HTML app + Excel)
Complete one-year + 3-year scenario planning tool for Sparkling Daily, delivered as a self-contained HTML app (11 views) and a matching 17-tab Excel workbook with identical, verified numbers. Custom scenarios, bulk edits, CSV import/export, portfolio mix, Summary one-pager, snapshot compare, Pricing Lab, Targets, Sensitivity (price and cost), Unit Economics, Monthly phasing with break-even month, and 3-Year projection. Auto-save, dark mode, keyboard shortcuts, accessibility, non-finite-safe. All figures are illustrative placeholders pending real inputs.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01QfvqvCPVnNVZ5knCrcjEgA
</commit_message>
<xml_diff>
--- a/Organika_Sparkling_Daily_1YR_Scenario_Model.xlsx
+++ b/Organika_Sparkling_Daily_1YR_Scenario_Model.xlsx
@@ -15,13 +15,15 @@
     <sheet name="High" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Stretch" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="Monthly" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Pricing Lab" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Targets" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Sensitivity" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Checks" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Guide" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Review Log" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Cover" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="3-Year" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Pricing Lab" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Unit Economics" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Targets" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Sensitivity" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Checks" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Guide" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Review Log" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Cover" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
     <definedName name="CP_Pineapple_Singles">'Assumptions'!$C$11</definedName>
@@ -215,7 +217,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="65">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -345,6 +347,12 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -1061,6 +1069,892 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
+  <dimension ref="B1:K21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="11" customWidth="1" min="6" max="6"/>
+    <col width="11" customWidth="1" min="7" max="7"/>
+    <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="11" customWidth="1" min="9" max="9"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>Sparkling Daily - Pricing Lab (FY2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>How wholesale price (CP) drives margin. Each column flexes every SKU's CP vs its Assumptions base; volume &amp; costs held at base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="48" t="inlineStr">
+        <is>
+          <t>Gross Profit %  (by SKU, by CP)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="17" t="inlineStr">
+        <is>
+          <t>SKU  \  CP vs base</t>
+        </is>
+      </c>
+      <c r="C5" s="49" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D5" s="49" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E5" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F5" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G5" s="49" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="H5" s="49" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="I5" s="49" t="n">
+        <v>1.15</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Pineapple Singles</t>
+        </is>
+      </c>
+      <c r="C6" s="39">
+        <f>IFERROR(1-'Assumptions'!$C$21/('Assumptions'!$C$11*C$5*(1-'Assumptions'!$C$12)),0)</f>
+        <v/>
+      </c>
+      <c r="D6" s="39">
+        <f>IFERROR(1-'Assumptions'!$C$21/('Assumptions'!$C$11*D$5*(1-'Assumptions'!$C$12)),0)</f>
+        <v/>
+      </c>
+      <c r="E6" s="39">
+        <f>IFERROR(1-'Assumptions'!$C$21/('Assumptions'!$C$11*E$5*(1-'Assumptions'!$C$12)),0)</f>
+        <v/>
+      </c>
+      <c r="F6" s="40">
+        <f>IFERROR(1-'Assumptions'!$C$21/('Assumptions'!$C$11*F$5*(1-'Assumptions'!$C$12)),0)</f>
+        <v/>
+      </c>
+      <c r="G6" s="39">
+        <f>IFERROR(1-'Assumptions'!$C$21/('Assumptions'!$C$11*G$5*(1-'Assumptions'!$C$12)),0)</f>
+        <v/>
+      </c>
+      <c r="H6" s="39">
+        <f>IFERROR(1-'Assumptions'!$C$21/('Assumptions'!$C$11*H$5*(1-'Assumptions'!$C$12)),0)</f>
+        <v/>
+      </c>
+      <c r="I6" s="39">
+        <f>IFERROR(1-'Assumptions'!$C$21/('Assumptions'!$C$11*I$5*(1-'Assumptions'!$C$12)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Passionfruit Singles</t>
+        </is>
+      </c>
+      <c r="C7" s="39">
+        <f>IFERROR(1-'Assumptions'!$D$21/('Assumptions'!$D$11*C$5*(1-'Assumptions'!$D$12)),0)</f>
+        <v/>
+      </c>
+      <c r="D7" s="39">
+        <f>IFERROR(1-'Assumptions'!$D$21/('Assumptions'!$D$11*D$5*(1-'Assumptions'!$D$12)),0)</f>
+        <v/>
+      </c>
+      <c r="E7" s="39">
+        <f>IFERROR(1-'Assumptions'!$D$21/('Assumptions'!$D$11*E$5*(1-'Assumptions'!$D$12)),0)</f>
+        <v/>
+      </c>
+      <c r="F7" s="40">
+        <f>IFERROR(1-'Assumptions'!$D$21/('Assumptions'!$D$11*F$5*(1-'Assumptions'!$D$12)),0)</f>
+        <v/>
+      </c>
+      <c r="G7" s="39">
+        <f>IFERROR(1-'Assumptions'!$D$21/('Assumptions'!$D$11*G$5*(1-'Assumptions'!$D$12)),0)</f>
+        <v/>
+      </c>
+      <c r="H7" s="39">
+        <f>IFERROR(1-'Assumptions'!$D$21/('Assumptions'!$D$11*H$5*(1-'Assumptions'!$D$12)),0)</f>
+        <v/>
+      </c>
+      <c r="I7" s="39">
+        <f>IFERROR(1-'Assumptions'!$D$21/('Assumptions'!$D$11*I$5*(1-'Assumptions'!$D$12)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Lime Lemon Singles</t>
+        </is>
+      </c>
+      <c r="C8" s="39">
+        <f>IFERROR(1-'Assumptions'!$E$21/('Assumptions'!$E$11*C$5*(1-'Assumptions'!$E$12)),0)</f>
+        <v/>
+      </c>
+      <c r="D8" s="39">
+        <f>IFERROR(1-'Assumptions'!$E$21/('Assumptions'!$E$11*D$5*(1-'Assumptions'!$E$12)),0)</f>
+        <v/>
+      </c>
+      <c r="E8" s="39">
+        <f>IFERROR(1-'Assumptions'!$E$21/('Assumptions'!$E$11*E$5*(1-'Assumptions'!$E$12)),0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="40">
+        <f>IFERROR(1-'Assumptions'!$E$21/('Assumptions'!$E$11*F$5*(1-'Assumptions'!$E$12)),0)</f>
+        <v/>
+      </c>
+      <c r="G8" s="39">
+        <f>IFERROR(1-'Assumptions'!$E$21/('Assumptions'!$E$11*G$5*(1-'Assumptions'!$E$12)),0)</f>
+        <v/>
+      </c>
+      <c r="H8" s="39">
+        <f>IFERROR(1-'Assumptions'!$E$21/('Assumptions'!$E$11*H$5*(1-'Assumptions'!$E$12)),0)</f>
+        <v/>
+      </c>
+      <c r="I8" s="39">
+        <f>IFERROR(1-'Assumptions'!$E$21/('Assumptions'!$E$11*I$5*(1-'Assumptions'!$E$12)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Pineapple 4-Pack</t>
+        </is>
+      </c>
+      <c r="C9" s="39">
+        <f>IFERROR(1-'Assumptions'!$F$21/('Assumptions'!$F$11*C$5*(1-'Assumptions'!$F$12)),0)</f>
+        <v/>
+      </c>
+      <c r="D9" s="39">
+        <f>IFERROR(1-'Assumptions'!$F$21/('Assumptions'!$F$11*D$5*(1-'Assumptions'!$F$12)),0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="39">
+        <f>IFERROR(1-'Assumptions'!$F$21/('Assumptions'!$F$11*E$5*(1-'Assumptions'!$F$12)),0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="40">
+        <f>IFERROR(1-'Assumptions'!$F$21/('Assumptions'!$F$11*F$5*(1-'Assumptions'!$F$12)),0)</f>
+        <v/>
+      </c>
+      <c r="G9" s="39">
+        <f>IFERROR(1-'Assumptions'!$F$21/('Assumptions'!$F$11*G$5*(1-'Assumptions'!$F$12)),0)</f>
+        <v/>
+      </c>
+      <c r="H9" s="39">
+        <f>IFERROR(1-'Assumptions'!$F$21/('Assumptions'!$F$11*H$5*(1-'Assumptions'!$F$12)),0)</f>
+        <v/>
+      </c>
+      <c r="I9" s="39">
+        <f>IFERROR(1-'Assumptions'!$F$21/('Assumptions'!$F$11*I$5*(1-'Assumptions'!$F$12)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Passionfruit 4-Pack</t>
+        </is>
+      </c>
+      <c r="C10" s="39">
+        <f>IFERROR(1-'Assumptions'!$G$21/('Assumptions'!$G$11*C$5*(1-'Assumptions'!$G$12)),0)</f>
+        <v/>
+      </c>
+      <c r="D10" s="39">
+        <f>IFERROR(1-'Assumptions'!$G$21/('Assumptions'!$G$11*D$5*(1-'Assumptions'!$G$12)),0)</f>
+        <v/>
+      </c>
+      <c r="E10" s="39">
+        <f>IFERROR(1-'Assumptions'!$G$21/('Assumptions'!$G$11*E$5*(1-'Assumptions'!$G$12)),0)</f>
+        <v/>
+      </c>
+      <c r="F10" s="40">
+        <f>IFERROR(1-'Assumptions'!$G$21/('Assumptions'!$G$11*F$5*(1-'Assumptions'!$G$12)),0)</f>
+        <v/>
+      </c>
+      <c r="G10" s="39">
+        <f>IFERROR(1-'Assumptions'!$G$21/('Assumptions'!$G$11*G$5*(1-'Assumptions'!$G$12)),0)</f>
+        <v/>
+      </c>
+      <c r="H10" s="39">
+        <f>IFERROR(1-'Assumptions'!$G$21/('Assumptions'!$G$11*H$5*(1-'Assumptions'!$G$12)),0)</f>
+        <v/>
+      </c>
+      <c r="I10" s="39">
+        <f>IFERROR(1-'Assumptions'!$G$21/('Assumptions'!$G$11*I$5*(1-'Assumptions'!$G$12)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Lime Lemon 4-Pack</t>
+        </is>
+      </c>
+      <c r="C11" s="39">
+        <f>IFERROR(1-'Assumptions'!$H$21/('Assumptions'!$H$11*C$5*(1-'Assumptions'!$H$12)),0)</f>
+        <v/>
+      </c>
+      <c r="D11" s="39">
+        <f>IFERROR(1-'Assumptions'!$H$21/('Assumptions'!$H$11*D$5*(1-'Assumptions'!$H$12)),0)</f>
+        <v/>
+      </c>
+      <c r="E11" s="39">
+        <f>IFERROR(1-'Assumptions'!$H$21/('Assumptions'!$H$11*E$5*(1-'Assumptions'!$H$12)),0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="40">
+        <f>IFERROR(1-'Assumptions'!$H$21/('Assumptions'!$H$11*F$5*(1-'Assumptions'!$H$12)),0)</f>
+        <v/>
+      </c>
+      <c r="G11" s="39">
+        <f>IFERROR(1-'Assumptions'!$H$21/('Assumptions'!$H$11*G$5*(1-'Assumptions'!$H$12)),0)</f>
+        <v/>
+      </c>
+      <c r="H11" s="39">
+        <f>IFERROR(1-'Assumptions'!$H$21/('Assumptions'!$H$11*H$5*(1-'Assumptions'!$H$12)),0)</f>
+        <v/>
+      </c>
+      <c r="I11" s="39">
+        <f>IFERROR(1-'Assumptions'!$H$21/('Assumptions'!$H$11*I$5*(1-'Assumptions'!$H$12)),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="48" t="inlineStr">
+        <is>
+          <t>Annual Contribution $  (by SKU, by CP — demand-adjusted)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>SKU  \  CP vs base</t>
+        </is>
+      </c>
+      <c r="C15" s="49" t="n">
+        <v>0.85</v>
+      </c>
+      <c r="D15" s="49" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="E15" s="49" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="F15" s="49" t="n">
+        <v>1</v>
+      </c>
+      <c r="G15" s="49" t="n">
+        <v>1.05</v>
+      </c>
+      <c r="H15" s="49" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="I15" s="49" t="n">
+        <v>1.15</v>
+      </c>
+      <c r="K15" s="18" t="inlineStr">
+        <is>
+          <t>Best CP ×</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Pineapple Singles</t>
+        </is>
+      </c>
+      <c r="C16" s="37">
+        <f>'Assumptions'!$C$28*(C$15^'Assumptions'!$C$39)*(('Assumptions'!$C$11*C$15*(1-'Assumptions'!$C$12))-'Assumptions'!$C$21-'Assumptions'!$C$26)</f>
+        <v/>
+      </c>
+      <c r="D16" s="37">
+        <f>'Assumptions'!$C$28*(D$15^'Assumptions'!$C$39)*(('Assumptions'!$C$11*D$15*(1-'Assumptions'!$C$12))-'Assumptions'!$C$21-'Assumptions'!$C$26)</f>
+        <v/>
+      </c>
+      <c r="E16" s="37">
+        <f>'Assumptions'!$C$28*(E$15^'Assumptions'!$C$39)*(('Assumptions'!$C$11*E$15*(1-'Assumptions'!$C$12))-'Assumptions'!$C$21-'Assumptions'!$C$26)</f>
+        <v/>
+      </c>
+      <c r="F16" s="38">
+        <f>'Assumptions'!$C$28*(F$15^'Assumptions'!$C$39)*(('Assumptions'!$C$11*F$15*(1-'Assumptions'!$C$12))-'Assumptions'!$C$21-'Assumptions'!$C$26)</f>
+        <v/>
+      </c>
+      <c r="G16" s="37">
+        <f>'Assumptions'!$C$28*(G$15^'Assumptions'!$C$39)*(('Assumptions'!$C$11*G$15*(1-'Assumptions'!$C$12))-'Assumptions'!$C$21-'Assumptions'!$C$26)</f>
+        <v/>
+      </c>
+      <c r="H16" s="37">
+        <f>'Assumptions'!$C$28*(H$15^'Assumptions'!$C$39)*(('Assumptions'!$C$11*H$15*(1-'Assumptions'!$C$12))-'Assumptions'!$C$21-'Assumptions'!$C$26)</f>
+        <v/>
+      </c>
+      <c r="I16" s="37">
+        <f>'Assumptions'!$C$28*(I$15^'Assumptions'!$C$39)*(('Assumptions'!$C$11*I$15*(1-'Assumptions'!$C$12))-'Assumptions'!$C$21-'Assumptions'!$C$26)</f>
+        <v/>
+      </c>
+      <c r="K16" s="50">
+        <f>INDEX($C$15:$I$15,MATCH(MAX(C16:I16),C16:I16,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Passionfruit Singles</t>
+        </is>
+      </c>
+      <c r="C17" s="37">
+        <f>'Assumptions'!$D$28*(C$15^'Assumptions'!$C$39)*(('Assumptions'!$D$11*C$15*(1-'Assumptions'!$D$12))-'Assumptions'!$D$21-'Assumptions'!$D$26)</f>
+        <v/>
+      </c>
+      <c r="D17" s="37">
+        <f>'Assumptions'!$D$28*(D$15^'Assumptions'!$C$39)*(('Assumptions'!$D$11*D$15*(1-'Assumptions'!$D$12))-'Assumptions'!$D$21-'Assumptions'!$D$26)</f>
+        <v/>
+      </c>
+      <c r="E17" s="37">
+        <f>'Assumptions'!$D$28*(E$15^'Assumptions'!$C$39)*(('Assumptions'!$D$11*E$15*(1-'Assumptions'!$D$12))-'Assumptions'!$D$21-'Assumptions'!$D$26)</f>
+        <v/>
+      </c>
+      <c r="F17" s="38">
+        <f>'Assumptions'!$D$28*(F$15^'Assumptions'!$C$39)*(('Assumptions'!$D$11*F$15*(1-'Assumptions'!$D$12))-'Assumptions'!$D$21-'Assumptions'!$D$26)</f>
+        <v/>
+      </c>
+      <c r="G17" s="37">
+        <f>'Assumptions'!$D$28*(G$15^'Assumptions'!$C$39)*(('Assumptions'!$D$11*G$15*(1-'Assumptions'!$D$12))-'Assumptions'!$D$21-'Assumptions'!$D$26)</f>
+        <v/>
+      </c>
+      <c r="H17" s="37">
+        <f>'Assumptions'!$D$28*(H$15^'Assumptions'!$C$39)*(('Assumptions'!$D$11*H$15*(1-'Assumptions'!$D$12))-'Assumptions'!$D$21-'Assumptions'!$D$26)</f>
+        <v/>
+      </c>
+      <c r="I17" s="37">
+        <f>'Assumptions'!$D$28*(I$15^'Assumptions'!$C$39)*(('Assumptions'!$D$11*I$15*(1-'Assumptions'!$D$12))-'Assumptions'!$D$21-'Assumptions'!$D$26)</f>
+        <v/>
+      </c>
+      <c r="K17" s="50">
+        <f>INDEX($C$15:$I$15,MATCH(MAX(C17:I17),C17:I17,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Lime Lemon Singles</t>
+        </is>
+      </c>
+      <c r="C18" s="37">
+        <f>'Assumptions'!$E$28*(C$15^'Assumptions'!$C$39)*(('Assumptions'!$E$11*C$15*(1-'Assumptions'!$E$12))-'Assumptions'!$E$21-'Assumptions'!$E$26)</f>
+        <v/>
+      </c>
+      <c r="D18" s="37">
+        <f>'Assumptions'!$E$28*(D$15^'Assumptions'!$C$39)*(('Assumptions'!$E$11*D$15*(1-'Assumptions'!$E$12))-'Assumptions'!$E$21-'Assumptions'!$E$26)</f>
+        <v/>
+      </c>
+      <c r="E18" s="37">
+        <f>'Assumptions'!$E$28*(E$15^'Assumptions'!$C$39)*(('Assumptions'!$E$11*E$15*(1-'Assumptions'!$E$12))-'Assumptions'!$E$21-'Assumptions'!$E$26)</f>
+        <v/>
+      </c>
+      <c r="F18" s="38">
+        <f>'Assumptions'!$E$28*(F$15^'Assumptions'!$C$39)*(('Assumptions'!$E$11*F$15*(1-'Assumptions'!$E$12))-'Assumptions'!$E$21-'Assumptions'!$E$26)</f>
+        <v/>
+      </c>
+      <c r="G18" s="37">
+        <f>'Assumptions'!$E$28*(G$15^'Assumptions'!$C$39)*(('Assumptions'!$E$11*G$15*(1-'Assumptions'!$E$12))-'Assumptions'!$E$21-'Assumptions'!$E$26)</f>
+        <v/>
+      </c>
+      <c r="H18" s="37">
+        <f>'Assumptions'!$E$28*(H$15^'Assumptions'!$C$39)*(('Assumptions'!$E$11*H$15*(1-'Assumptions'!$E$12))-'Assumptions'!$E$21-'Assumptions'!$E$26)</f>
+        <v/>
+      </c>
+      <c r="I18" s="37">
+        <f>'Assumptions'!$E$28*(I$15^'Assumptions'!$C$39)*(('Assumptions'!$E$11*I$15*(1-'Assumptions'!$E$12))-'Assumptions'!$E$21-'Assumptions'!$E$26)</f>
+        <v/>
+      </c>
+      <c r="K18" s="50">
+        <f>INDEX($C$15:$I$15,MATCH(MAX(C18:I18),C18:I18,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Pineapple 4-Pack</t>
+        </is>
+      </c>
+      <c r="C19" s="37">
+        <f>'Assumptions'!$F$28*(C$15^'Assumptions'!$C$39)*(('Assumptions'!$F$11*C$15*(1-'Assumptions'!$F$12))-'Assumptions'!$F$21-'Assumptions'!$F$26)</f>
+        <v/>
+      </c>
+      <c r="D19" s="37">
+        <f>'Assumptions'!$F$28*(D$15^'Assumptions'!$C$39)*(('Assumptions'!$F$11*D$15*(1-'Assumptions'!$F$12))-'Assumptions'!$F$21-'Assumptions'!$F$26)</f>
+        <v/>
+      </c>
+      <c r="E19" s="37">
+        <f>'Assumptions'!$F$28*(E$15^'Assumptions'!$C$39)*(('Assumptions'!$F$11*E$15*(1-'Assumptions'!$F$12))-'Assumptions'!$F$21-'Assumptions'!$F$26)</f>
+        <v/>
+      </c>
+      <c r="F19" s="38">
+        <f>'Assumptions'!$F$28*(F$15^'Assumptions'!$C$39)*(('Assumptions'!$F$11*F$15*(1-'Assumptions'!$F$12))-'Assumptions'!$F$21-'Assumptions'!$F$26)</f>
+        <v/>
+      </c>
+      <c r="G19" s="37">
+        <f>'Assumptions'!$F$28*(G$15^'Assumptions'!$C$39)*(('Assumptions'!$F$11*G$15*(1-'Assumptions'!$F$12))-'Assumptions'!$F$21-'Assumptions'!$F$26)</f>
+        <v/>
+      </c>
+      <c r="H19" s="37">
+        <f>'Assumptions'!$F$28*(H$15^'Assumptions'!$C$39)*(('Assumptions'!$F$11*H$15*(1-'Assumptions'!$F$12))-'Assumptions'!$F$21-'Assumptions'!$F$26)</f>
+        <v/>
+      </c>
+      <c r="I19" s="37">
+        <f>'Assumptions'!$F$28*(I$15^'Assumptions'!$C$39)*(('Assumptions'!$F$11*I$15*(1-'Assumptions'!$F$12))-'Assumptions'!$F$21-'Assumptions'!$F$26)</f>
+        <v/>
+      </c>
+      <c r="K19" s="50">
+        <f>INDEX($C$15:$I$15,MATCH(MAX(C19:I19),C19:I19,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Passionfruit 4-Pack</t>
+        </is>
+      </c>
+      <c r="C20" s="37">
+        <f>'Assumptions'!$G$28*(C$15^'Assumptions'!$C$39)*(('Assumptions'!$G$11*C$15*(1-'Assumptions'!$G$12))-'Assumptions'!$G$21-'Assumptions'!$G$26)</f>
+        <v/>
+      </c>
+      <c r="D20" s="37">
+        <f>'Assumptions'!$G$28*(D$15^'Assumptions'!$C$39)*(('Assumptions'!$G$11*D$15*(1-'Assumptions'!$G$12))-'Assumptions'!$G$21-'Assumptions'!$G$26)</f>
+        <v/>
+      </c>
+      <c r="E20" s="37">
+        <f>'Assumptions'!$G$28*(E$15^'Assumptions'!$C$39)*(('Assumptions'!$G$11*E$15*(1-'Assumptions'!$G$12))-'Assumptions'!$G$21-'Assumptions'!$G$26)</f>
+        <v/>
+      </c>
+      <c r="F20" s="38">
+        <f>'Assumptions'!$G$28*(F$15^'Assumptions'!$C$39)*(('Assumptions'!$G$11*F$15*(1-'Assumptions'!$G$12))-'Assumptions'!$G$21-'Assumptions'!$G$26)</f>
+        <v/>
+      </c>
+      <c r="G20" s="37">
+        <f>'Assumptions'!$G$28*(G$15^'Assumptions'!$C$39)*(('Assumptions'!$G$11*G$15*(1-'Assumptions'!$G$12))-'Assumptions'!$G$21-'Assumptions'!$G$26)</f>
+        <v/>
+      </c>
+      <c r="H20" s="37">
+        <f>'Assumptions'!$G$28*(H$15^'Assumptions'!$C$39)*(('Assumptions'!$G$11*H$15*(1-'Assumptions'!$G$12))-'Assumptions'!$G$21-'Assumptions'!$G$26)</f>
+        <v/>
+      </c>
+      <c r="I20" s="37">
+        <f>'Assumptions'!$G$28*(I$15^'Assumptions'!$C$39)*(('Assumptions'!$G$11*I$15*(1-'Assumptions'!$G$12))-'Assumptions'!$G$21-'Assumptions'!$G$26)</f>
+        <v/>
+      </c>
+      <c r="K20" s="50">
+        <f>INDEX($C$15:$I$15,MATCH(MAX(C20:I20),C20:I20,0))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Lime Lemon 4-Pack</t>
+        </is>
+      </c>
+      <c r="C21" s="37">
+        <f>'Assumptions'!$H$28*(C$15^'Assumptions'!$C$39)*(('Assumptions'!$H$11*C$15*(1-'Assumptions'!$H$12))-'Assumptions'!$H$21-'Assumptions'!$H$26)</f>
+        <v/>
+      </c>
+      <c r="D21" s="37">
+        <f>'Assumptions'!$H$28*(D$15^'Assumptions'!$C$39)*(('Assumptions'!$H$11*D$15*(1-'Assumptions'!$H$12))-'Assumptions'!$H$21-'Assumptions'!$H$26)</f>
+        <v/>
+      </c>
+      <c r="E21" s="37">
+        <f>'Assumptions'!$H$28*(E$15^'Assumptions'!$C$39)*(('Assumptions'!$H$11*E$15*(1-'Assumptions'!$H$12))-'Assumptions'!$H$21-'Assumptions'!$H$26)</f>
+        <v/>
+      </c>
+      <c r="F21" s="38">
+        <f>'Assumptions'!$H$28*(F$15^'Assumptions'!$C$39)*(('Assumptions'!$H$11*F$15*(1-'Assumptions'!$H$12))-'Assumptions'!$H$21-'Assumptions'!$H$26)</f>
+        <v/>
+      </c>
+      <c r="G21" s="37">
+        <f>'Assumptions'!$H$28*(G$15^'Assumptions'!$C$39)*(('Assumptions'!$H$11*G$15*(1-'Assumptions'!$H$12))-'Assumptions'!$H$21-'Assumptions'!$H$26)</f>
+        <v/>
+      </c>
+      <c r="H21" s="37">
+        <f>'Assumptions'!$H$28*(H$15^'Assumptions'!$C$39)*(('Assumptions'!$H$11*H$15*(1-'Assumptions'!$H$12))-'Assumptions'!$H$21-'Assumptions'!$H$26)</f>
+        <v/>
+      </c>
+      <c r="I21" s="37">
+        <f>'Assumptions'!$H$28*(I$15^'Assumptions'!$C$39)*(('Assumptions'!$H$11*I$15*(1-'Assumptions'!$H$12))-'Assumptions'!$H$21-'Assumptions'!$H$26)</f>
+        <v/>
+      </c>
+      <c r="K21" s="50">
+        <f>INDEX($C$15:$I$15,MATCH(MAX(C21:I21),C21:I21,0))</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;LSparkling Daily • FY2026&amp;C&amp;A&amp;Rv2.0 • Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="006A1B9A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="B1:H13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="13" customWidth="1" min="3" max="3"/>
+    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="13" customWidth="1" min="8" max="8"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="B1" s="14" t="inlineStr">
+        <is>
+          <t>Sparkling Daily - Unit Economics &amp; Retail Price (FY2026)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="B2" s="15" t="inlineStr">
+        <is>
+          <t>Per-unit view of each SKU, plus the suggested shelf price at your retailer's margin.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>Retailer margin</t>
+        </is>
+      </c>
+      <c r="C4" s="26" t="n">
+        <v>0.35</v>
+      </c>
+      <c r="D4" s="45" t="inlineStr">
+        <is>
+          <t>shelf price = wholesale unit price / (1 - margin)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="17" t="inlineStr">
+        <is>
+          <t>Per unit (CDN $)</t>
+        </is>
+      </c>
+      <c r="C6" s="18" t="inlineStr">
+        <is>
+          <t>Pineapple</t>
+        </is>
+      </c>
+      <c r="D6" s="18" t="inlineStr">
+        <is>
+          <t>Passionfruit</t>
+        </is>
+      </c>
+      <c r="E6" s="18" t="inlineStr">
+        <is>
+          <t>Lime Lemon</t>
+        </is>
+      </c>
+      <c r="F6" s="18" t="inlineStr">
+        <is>
+          <t>Pineapple</t>
+        </is>
+      </c>
+      <c r="G6" s="18" t="inlineStr">
+        <is>
+          <t>Passionfruit</t>
+        </is>
+      </c>
+      <c r="H6" s="18" t="inlineStr">
+        <is>
+          <t>Lime Lemon</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Units per case</t>
+        </is>
+      </c>
+      <c r="C7" s="36">
+        <f>'Assumptions'!C9</f>
+        <v/>
+      </c>
+      <c r="D7" s="36">
+        <f>'Assumptions'!D9</f>
+        <v/>
+      </c>
+      <c r="E7" s="36">
+        <f>'Assumptions'!E9</f>
+        <v/>
+      </c>
+      <c r="F7" s="36">
+        <f>'Assumptions'!F9</f>
+        <v/>
+      </c>
+      <c r="G7" s="36">
+        <f>'Assumptions'!G9</f>
+        <v/>
+      </c>
+      <c r="H7" s="36">
+        <f>'Assumptions'!H9</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Wholesale (CP) / unit</t>
+        </is>
+      </c>
+      <c r="C8" s="27">
+        <f>IFERROR('Assumptions'!C11/'Assumptions'!C9,0)</f>
+        <v/>
+      </c>
+      <c r="D8" s="27">
+        <f>IFERROR('Assumptions'!D11/'Assumptions'!D9,0)</f>
+        <v/>
+      </c>
+      <c r="E8" s="27">
+        <f>IFERROR('Assumptions'!E11/'Assumptions'!E9,0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="27">
+        <f>IFERROR('Assumptions'!F11/'Assumptions'!F9,0)</f>
+        <v/>
+      </c>
+      <c r="G8" s="27">
+        <f>IFERROR('Assumptions'!G11/'Assumptions'!G9,0)</f>
+        <v/>
+      </c>
+      <c r="H8" s="27">
+        <f>IFERROR('Assumptions'!H11/'Assumptions'!H9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Net / unit (after disc)</t>
+        </is>
+      </c>
+      <c r="C9" s="27">
+        <f>IFERROR('Assumptions'!C11*(1-'Assumptions'!C12)/'Assumptions'!C9,0)</f>
+        <v/>
+      </c>
+      <c r="D9" s="27">
+        <f>IFERROR('Assumptions'!D11*(1-'Assumptions'!D12)/'Assumptions'!D9,0)</f>
+        <v/>
+      </c>
+      <c r="E9" s="27">
+        <f>IFERROR('Assumptions'!E11*(1-'Assumptions'!E12)/'Assumptions'!E9,0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="27">
+        <f>IFERROR('Assumptions'!F11*(1-'Assumptions'!F12)/'Assumptions'!F9,0)</f>
+        <v/>
+      </c>
+      <c r="G9" s="27">
+        <f>IFERROR('Assumptions'!G11*(1-'Assumptions'!G12)/'Assumptions'!G9,0)</f>
+        <v/>
+      </c>
+      <c r="H9" s="27">
+        <f>IFERROR('Assumptions'!H11*(1-'Assumptions'!H12)/'Assumptions'!H9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   COGS / unit</t>
+        </is>
+      </c>
+      <c r="C10" s="27">
+        <f>IFERROR('Assumptions'!C21/'Assumptions'!C9,0)</f>
+        <v/>
+      </c>
+      <c r="D10" s="27">
+        <f>IFERROR('Assumptions'!D21/'Assumptions'!D9,0)</f>
+        <v/>
+      </c>
+      <c r="E10" s="27">
+        <f>IFERROR('Assumptions'!E21/'Assumptions'!E9,0)</f>
+        <v/>
+      </c>
+      <c r="F10" s="27">
+        <f>IFERROR('Assumptions'!F21/'Assumptions'!F9,0)</f>
+        <v/>
+      </c>
+      <c r="G10" s="27">
+        <f>IFERROR('Assumptions'!G21/'Assumptions'!G9,0)</f>
+        <v/>
+      </c>
+      <c r="H10" s="27">
+        <f>IFERROR('Assumptions'!H21/'Assumptions'!H9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="B11" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Gross profit / unit</t>
+        </is>
+      </c>
+      <c r="C11" s="28">
+        <f>C9-C10</f>
+        <v/>
+      </c>
+      <c r="D11" s="28">
+        <f>D9-D10</f>
+        <v/>
+      </c>
+      <c r="E11" s="28">
+        <f>E9-E10</f>
+        <v/>
+      </c>
+      <c r="F11" s="28">
+        <f>F9-F10</f>
+        <v/>
+      </c>
+      <c r="G11" s="28">
+        <f>G9-G10</f>
+        <v/>
+      </c>
+      <c r="H11" s="28">
+        <f>H9-H10</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   GP %</t>
+        </is>
+      </c>
+      <c r="C12" s="40">
+        <f>IFERROR(C11/C9,0)</f>
+        <v/>
+      </c>
+      <c r="D12" s="40">
+        <f>IFERROR(D11/D9,0)</f>
+        <v/>
+      </c>
+      <c r="E12" s="40">
+        <f>IFERROR(E11/E9,0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="40">
+        <f>IFERROR(F11/F9,0)</f>
+        <v/>
+      </c>
+      <c r="G12" s="40">
+        <f>IFERROR(G11/G9,0)</f>
+        <v/>
+      </c>
+      <c r="H12" s="40">
+        <f>IFERROR(H11/H9,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Suggested shelf / unit</t>
+        </is>
+      </c>
+      <c r="C13" s="28">
+        <f>IFERROR(C8/(1-$C$4),0)</f>
+        <v/>
+      </c>
+      <c r="D13" s="28">
+        <f>IFERROR(D8/(1-$C$4),0)</f>
+        <v/>
+      </c>
+      <c r="E13" s="28">
+        <f>IFERROR(E8/(1-$C$4),0)</f>
+        <v/>
+      </c>
+      <c r="F13" s="28">
+        <f>IFERROR(F8/(1-$C$4),0)</f>
+        <v/>
+      </c>
+      <c r="G13" s="28">
+        <f>IFERROR(G8/(1-$C$4),0)</f>
+        <v/>
+      </c>
+      <c r="H13" s="28">
+        <f>IFERROR(H8/(1-$C$4),0)</f>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;LSparkling Daily • FY2026&amp;C&amp;A&amp;Rv2.0 • Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <tabColor rgb="006A1B9A"/>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="B1:C24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -1084,7 +1978,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="46" t="inlineStr">
+      <c r="B4" s="48" t="inlineStr">
         <is>
           <t>Model constants (from Assumptions)</t>
         </is>
@@ -1157,7 +2051,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="46" t="inlineStr">
+      <c r="B13" s="48" t="inlineStr">
         <is>
           <t>Your targets (edit yellow)</t>
         </is>
@@ -1184,7 +2078,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="46" t="inlineStr">
+      <c r="B17" s="48" t="inlineStr">
         <is>
           <t>Solved answers</t>
         </is>
@@ -1196,7 +2090,7 @@
           <t xml:space="preserve">   Price × to hit target GP % (base volume)</t>
         </is>
       </c>
-      <c r="C18" s="49">
+      <c r="C18" s="51">
         <f>IFERROR($C$6/($C$5*(1-$C$14)),"n/a")</f>
         <v/>
       </c>
@@ -1218,7 +2112,7 @@
           <t xml:space="preserve">   Volume × to hit target EBITDA (base price)</t>
         </is>
       </c>
-      <c r="C20" s="49">
+      <c r="C20" s="51">
         <f>IFERROR(($C$15+$C$8)/(($C$5-$C$6-$C$7)-$C$9*$C$5),"n/a")</f>
         <v/>
       </c>
@@ -1240,7 +2134,7 @@
           <t xml:space="preserve">   Price × to hit target EBITDA (base vol; ε=0 approx)</t>
         </is>
       </c>
-      <c r="C22" s="49">
+      <c r="C22" s="51">
         <f>IFERROR(($C$15+$C$8+$C$6+$C$7)/($C$5*(1-$C$9)),"n/a")</f>
         <v/>
       </c>
@@ -1251,7 +2145,7 @@
           <t xml:space="preserve">   Break-even volume × (EBITDA = 0, base price)</t>
         </is>
       </c>
-      <c r="C23" s="49">
+      <c r="C23" s="51">
         <f>IFERROR($C$8/(($C$5-$C$6-$C$7)-$C$9*$C$5),"n/a")</f>
         <v/>
       </c>
@@ -1281,7 +2175,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00EF6C00"/>
@@ -1377,13 +2271,13 @@
           <t>Price elasticity (from Assumptions)</t>
         </is>
       </c>
-      <c r="C9" s="50">
+      <c r="C9" s="52">
         <f>'Assumptions'!C39</f>
         <v/>
       </c>
     </row>
     <row r="11">
-      <c r="B11" s="46" t="inlineStr">
+      <c r="B11" s="48" t="inlineStr">
         <is>
           <t>EBITDA  ($)</t>
         </is>
@@ -1395,30 +2289,30 @@
           <t>Price x  \  Volume x</t>
         </is>
       </c>
-      <c r="C12" s="47" t="n">
+      <c r="C12" s="49" t="n">
         <v>0.7</v>
       </c>
-      <c r="D12" s="47" t="n">
+      <c r="D12" s="49" t="n">
         <v>0.9</v>
       </c>
-      <c r="E12" s="47" t="n">
+      <c r="E12" s="49" t="n">
         <v>1</v>
       </c>
-      <c r="F12" s="47" t="n">
+      <c r="F12" s="49" t="n">
         <v>1.1</v>
       </c>
-      <c r="G12" s="47" t="n">
+      <c r="G12" s="49" t="n">
         <v>1.3</v>
       </c>
-      <c r="H12" s="47" t="n">
+      <c r="H12" s="49" t="n">
         <v>1.5</v>
       </c>
-      <c r="I12" s="47" t="n">
+      <c r="I12" s="49" t="n">
         <v>1.7</v>
       </c>
     </row>
     <row r="13">
-      <c r="B13" s="47" t="n">
+      <c r="B13" s="49" t="n">
         <v>0.9</v>
       </c>
       <c r="C13" s="37">
@@ -1451,7 +2345,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="47" t="n">
+      <c r="B14" s="49" t="n">
         <v>0.95</v>
       </c>
       <c r="C14" s="37">
@@ -1484,7 +2378,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="47" t="n">
+      <c r="B15" s="49" t="n">
         <v>1</v>
       </c>
       <c r="C15" s="37">
@@ -1517,7 +2411,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="47" t="n">
+      <c r="B16" s="49" t="n">
         <v>1.05</v>
       </c>
       <c r="C16" s="37">
@@ -1550,7 +2444,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="47" t="n">
+      <c r="B17" s="49" t="n">
         <v>1.1</v>
       </c>
       <c r="C17" s="37">
@@ -1583,7 +2477,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="47" t="n">
+      <c r="B18" s="49" t="n">
         <v>1.15</v>
       </c>
       <c r="C18" s="37">
@@ -1616,7 +2510,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="46" t="inlineStr">
+      <c r="B21" s="48" t="inlineStr">
         <is>
           <t>BREAK-EVEN (at Base price)</t>
         </is>
@@ -1628,7 +2522,7 @@
           <t>Volume x for EBITDA = 0</t>
         </is>
       </c>
-      <c r="C22" s="49">
+      <c r="C22" s="51">
         <f>IFERROR($C$6/(($C$4-$C$5)-$C$7*$C$4),0)</f>
         <v/>
       </c>
@@ -1669,7 +2563,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00B00020"/>
@@ -1723,11 +2617,11 @@
         </is>
       </c>
       <c r="C5" s="39">
-        <f>SUM('Assumptions'!C50:N50)</f>
-        <v/>
-      </c>
-      <c r="D5" s="51">
-        <f>IF(ABS(SUM('Assumptions'!C50:N50)-1)&lt;0.0001,"PASS","FAIL")</f>
+        <f>SUM('Assumptions'!C53:N53)</f>
+        <v/>
+      </c>
+      <c r="D5" s="53">
+        <f>IF(ABS(SUM('Assumptions'!C53:N53)-1)&lt;0.0001,"PASS","FAIL")</f>
         <v/>
       </c>
     </row>
@@ -1741,7 +2635,7 @@
         <f>MIN('Assumptions'!C11:H11)</f>
         <v/>
       </c>
-      <c r="D6" s="51">
+      <c r="D6" s="53">
         <f>IF(MIN('Assumptions'!C11:H11)&gt;0,"PASS","FAIL")</f>
         <v/>
       </c>
@@ -1756,7 +2650,7 @@
         <f>MIN('Assumptions'!C28:H28)</f>
         <v/>
       </c>
-      <c r="D7" s="51">
+      <c r="D7" s="53">
         <f>IF(MIN('Assumptions'!C28:H28)&gt;=0,"PASS","FAIL")</f>
         <v/>
       </c>
@@ -1771,7 +2665,7 @@
         <f>MAX('Assumptions'!C12:H12)</f>
         <v/>
       </c>
-      <c r="D8" s="51">
+      <c r="D8" s="53">
         <f>IF(AND(MIN('Assumptions'!C12:H12)&gt;=0,MAX('Assumptions'!C12:H12)&lt;=0.5),"PASS","FAIL")</f>
         <v/>
       </c>
@@ -1786,7 +2680,7 @@
         <f>'Base'!I23</f>
         <v/>
       </c>
-      <c r="D9" s="51">
+      <c r="D9" s="53">
         <f>IF(AND('Base'!I23&gt;0,'Base'!I23&lt;1),"PASS","FAIL")</f>
         <v/>
       </c>
@@ -1801,7 +2695,7 @@
         <f>SUMPRODUCT(--('Assumptions'!C19:H19&gt;='Assumptions'!C11:H11))</f>
         <v/>
       </c>
-      <c r="D10" s="51">
+      <c r="D10" s="53">
         <f>IF(SUMPRODUCT(--('Assumptions'!C19:H19&gt;='Assumptions'!C11:H11))=0,"PASS","FAIL")</f>
         <v/>
       </c>
@@ -1816,7 +2710,7 @@
         <f>'Assumptions'!C38</f>
         <v/>
       </c>
-      <c r="D11" s="51">
+      <c r="D11" s="53">
         <f>IF(AND('Assumptions'!C38&gt;=0,'Assumptions'!C38&lt;=0.5),"PASS","FAIL")</f>
         <v/>
       </c>
@@ -1827,12 +2721,12 @@
           <t>All scenario volume levers &gt; 0</t>
         </is>
       </c>
-      <c r="C12" s="52">
-        <f>MIN('Assumptions'!C43:C46)</f>
-        <v/>
-      </c>
-      <c r="D12" s="51">
-        <f>IF(MIN('Assumptions'!C43:C46)&gt;0,"PASS","FAIL")</f>
+      <c r="C12" s="54">
+        <f>MIN('Assumptions'!C46:C49)</f>
+        <v/>
+      </c>
+      <c r="D12" s="53">
+        <f>IF(MIN('Assumptions'!C46:C49)&gt;0,"PASS","FAIL")</f>
         <v/>
       </c>
     </row>
@@ -1842,11 +2736,11 @@
           <t>Price elasticity &lt;= 0 (demand sane)</t>
         </is>
       </c>
-      <c r="C13" s="53">
+      <c r="C13" s="55">
         <f>'Assumptions'!C39</f>
         <v/>
       </c>
-      <c r="D13" s="51">
+      <c r="D13" s="53">
         <f>IF('Assumptions'!C39&lt;=0,"PASS","FAIL")</f>
         <v/>
       </c>
@@ -1861,7 +2755,7 @@
         <f>'Dashboard'!D8-'Base'!I18</f>
         <v/>
       </c>
-      <c r="D14" s="51">
+      <c r="D14" s="53">
         <f>IF(ABS('Dashboard'!D8-'Base'!I18)&lt;1,"PASS","FAIL")</f>
         <v/>
       </c>
@@ -1872,7 +2766,7 @@
           <t>OVERALL</t>
         </is>
       </c>
-      <c r="D16" s="51">
+      <c r="D16" s="53">
         <f>IF(COUNTIF(D5:D14,"FAIL")=0,"ALL PASS","REVIEW")</f>
         <v/>
       </c>
@@ -1899,7 +2793,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00808A99"/>
@@ -1914,14 +2808,14 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="B1" s="54" t="inlineStr">
+      <c r="B1" s="56" t="inlineStr">
         <is>
           <t>Sparkling Daily — Model Guide</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="B2" s="55" t="inlineStr"/>
+      <c r="B2" s="57" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="B3" s="24" t="inlineStr">
@@ -1959,7 +2853,7 @@
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="55" t="inlineStr"/>
+      <c r="B8" s="57" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="B9" s="24" t="inlineStr">
@@ -1983,7 +2877,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="B12" s="55" t="inlineStr"/>
+      <c r="B12" s="57" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="B13" s="24" t="inlineStr">
@@ -2028,7 +2922,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="55" t="inlineStr"/>
+      <c r="B19" s="57" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="B20" s="24" t="inlineStr">
@@ -2080,7 +2974,7 @@
       </c>
     </row>
     <row r="27">
-      <c r="B27" s="55" t="inlineStr"/>
+      <c r="B27" s="57" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="B28" s="24" t="inlineStr">
@@ -2132,7 +3026,7 @@
       </c>
     </row>
     <row r="35">
-      <c r="B35" s="55" t="inlineStr"/>
+      <c r="B35" s="57" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="B36" s="24" t="inlineStr">
@@ -2169,7 +3063,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00808A99"/>
@@ -2226,17 +3120,17 @@
       <c r="B5" s="22" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="56" t="inlineStr">
+      <c r="C5" s="58" t="inlineStr">
         <is>
           <t>No single source of truth — costs hand-keyed in ~24 places across tabs.</t>
         </is>
       </c>
-      <c r="D5" s="56" t="inlineStr">
+      <c r="D5" s="58" t="inlineStr">
         <is>
           <t>Added Assumptions tab; all scenarios/monthly/sensitivity read from it (DRY).</t>
         </is>
       </c>
-      <c r="E5" s="51" t="inlineStr">
+      <c r="E5" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2246,17 +3140,17 @@
       <c r="B6" s="22" t="n">
         <v>2</v>
       </c>
-      <c r="C6" s="56" t="inlineStr">
+      <c r="C6" s="58" t="inlineStr">
         <is>
           <t>Trade discount modelled as flat $/case — unrealistic.</t>
         </is>
       </c>
-      <c r="D6" s="56" t="inlineStr">
+      <c r="D6" s="58" t="inlineStr">
         <is>
           <t>Now % of gross revenue, per SKU, flexed by scenario.</t>
         </is>
       </c>
-      <c r="E6" s="51" t="inlineStr">
+      <c r="E6" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2266,17 +3160,17 @@
       <c r="B7" s="22" t="n">
         <v>3</v>
       </c>
-      <c r="C7" s="56" t="inlineStr">
+      <c r="C7" s="58" t="inlineStr">
         <is>
           <t>COGS was a single lump — no cost visibility.</t>
         </is>
       </c>
-      <c r="D7" s="56" t="inlineStr">
+      <c r="D7" s="58" t="inlineStr">
         <is>
           <t>Built up from ingredients, packaging, co-pack, inbound freight + warehousing.</t>
         </is>
       </c>
-      <c r="E7" s="51" t="inlineStr">
+      <c r="E7" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2286,17 +3180,17 @@
       <c r="B8" s="22" t="n">
         <v>4</v>
       </c>
-      <c r="C8" s="56" t="inlineStr">
+      <c r="C8" s="58" t="inlineStr">
         <is>
           <t>P&amp;L stopped at contribution — not a real P&amp;L.</t>
         </is>
       </c>
-      <c r="D8" s="56" t="inlineStr">
+      <c r="D8" s="58" t="inlineStr">
         <is>
           <t>Extended to Opex → EBITDA → EBIT → Pre-tax → Net Income.</t>
         </is>
       </c>
-      <c r="E8" s="51" t="inlineStr">
+      <c r="E8" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2306,17 +3200,17 @@
       <c r="B9" s="22" t="n">
         <v>5</v>
       </c>
-      <c r="C9" s="56" t="inlineStr">
+      <c r="C9" s="58" t="inlineStr">
         <is>
           <t>No operating leverage — all costs implicitly variable.</t>
         </is>
       </c>
-      <c r="D9" s="56" t="inlineStr">
+      <c r="D9" s="58" t="inlineStr">
         <is>
           <t>Split fixed (salaries/G&amp;A/mktg/slotting) vs variable (logistics % of net).</t>
         </is>
       </c>
-      <c r="E9" s="51" t="inlineStr">
+      <c r="E9" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2326,17 +3220,17 @@
       <c r="B10" s="22" t="n">
         <v>6</v>
       </c>
-      <c r="C10" s="56" t="inlineStr">
+      <c r="C10" s="58" t="inlineStr">
         <is>
           <t>Annual only — no phasing.</t>
         </is>
       </c>
-      <c r="D10" s="56" t="inlineStr">
+      <c r="D10" s="58" t="inlineStr">
         <is>
           <t>Added Monthly tab driven by a seasonality curve.</t>
         </is>
       </c>
-      <c r="E10" s="51" t="inlineStr">
+      <c r="E10" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2346,17 +3240,17 @@
       <c r="B11" s="22" t="n">
         <v>7</v>
       </c>
-      <c r="C11" s="56" t="inlineStr">
+      <c r="C11" s="58" t="inlineStr">
         <is>
           <t>No way to switch scenario in one view.</t>
         </is>
       </c>
-      <c r="D11" s="56" t="inlineStr">
+      <c r="D11" s="58" t="inlineStr">
         <is>
           <t>Monthly has a dropdown selector (INDIRECT-driven).</t>
         </is>
       </c>
-      <c r="E11" s="51" t="inlineStr">
+      <c r="E11" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2366,17 +3260,17 @@
       <c r="B12" s="22" t="n">
         <v>8</v>
       </c>
-      <c r="C12" s="56" t="inlineStr">
+      <c r="C12" s="58" t="inlineStr">
         <is>
           <t>No sensitivity or break-even.</t>
         </is>
       </c>
-      <c r="D12" s="56" t="inlineStr">
+      <c r="D12" s="58" t="inlineStr">
         <is>
           <t>Two-way EBITDA table (price × volume) + break-even volume, closed-form.</t>
         </is>
       </c>
-      <c r="E12" s="51" t="inlineStr">
+      <c r="E12" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2386,17 +3280,17 @@
       <c r="B13" s="22" t="n">
         <v>9</v>
       </c>
-      <c r="C13" s="56" t="inlineStr">
+      <c r="C13" s="58" t="inlineStr">
         <is>
           <t>No validation of inputs/outputs.</t>
         </is>
       </c>
-      <c r="D13" s="56" t="inlineStr">
+      <c r="D13" s="58" t="inlineStr">
         <is>
           <t>Checks tab with PASS/FAIL incl. a tie-out of Dashboard to Base.</t>
         </is>
       </c>
-      <c r="E13" s="51" t="inlineStr">
+      <c r="E13" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2406,17 +3300,17 @@
       <c r="B14" s="22" t="n">
         <v>10</v>
       </c>
-      <c r="C14" s="56" t="inlineStr">
+      <c r="C14" s="58" t="inlineStr">
         <is>
           <t>No governance / context.</t>
         </is>
       </c>
-      <c r="D14" s="56" t="inlineStr">
+      <c r="D14" s="58" t="inlineStr">
         <is>
           <t>Cover (purpose, version, owner, legend), Guide + glossary, this Review Log.</t>
         </is>
       </c>
-      <c r="E14" s="51" t="inlineStr">
+      <c r="E14" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2426,17 +3320,17 @@
       <c r="B15" s="22" t="n">
         <v>11</v>
       </c>
-      <c r="C15" s="56" t="inlineStr">
+      <c r="C15" s="58" t="inlineStr">
         <is>
           <t>Tax could show a fictitious credit on losses.</t>
         </is>
       </c>
-      <c r="D15" s="56" t="inlineStr">
+      <c r="D15" s="58" t="inlineStr">
         <is>
           <t>Tax floored at 0 via MAX(0, EBT×rate).</t>
         </is>
       </c>
-      <c r="E15" s="51" t="inlineStr">
+      <c r="E15" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2446,17 +3340,17 @@
       <c r="B16" s="22" t="n">
         <v>12</v>
       </c>
-      <c r="C16" s="56" t="inlineStr">
+      <c r="C16" s="58" t="inlineStr">
         <is>
           <t>Inputs vs calcs indistinguishable.</t>
         </is>
       </c>
-      <c r="D16" s="56" t="inlineStr">
+      <c r="D16" s="58" t="inlineStr">
         <is>
           <t>Colour coding: yellow = input, blue tint = calculated total; freeze panes throughout.</t>
         </is>
       </c>
-      <c r="E16" s="51" t="inlineStr">
+      <c r="E16" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2466,17 +3360,17 @@
       <c r="B17" s="22" t="n">
         <v>13</v>
       </c>
-      <c r="C17" s="56" t="inlineStr">
+      <c r="C17" s="58" t="inlineStr">
         <is>
           <t>Flavour names were placeholders.</t>
         </is>
       </c>
-      <c r="D17" s="56" t="inlineStr">
+      <c r="D17" s="58" t="inlineStr">
         <is>
           <t>Set to Pineapple, Passionfruit, Lime Lemon (editable on Assumptions).</t>
         </is>
       </c>
-      <c r="E17" s="51" t="inlineStr">
+      <c r="E17" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2486,17 +3380,17 @@
       <c r="B18" s="22" t="n">
         <v>14</v>
       </c>
-      <c r="C18" s="56" t="inlineStr">
+      <c r="C18" s="58" t="inlineStr">
         <is>
           <t>Price and volume were independent — raising CP with no volume loss is unrealistic.</t>
         </is>
       </c>
-      <c r="D18" s="56" t="inlineStr">
+      <c r="D18" s="58" t="inlineStr">
         <is>
           <t>Added optional price elasticity; volume now responds to price. Pricing Lab finds the best CP.</t>
         </is>
       </c>
-      <c r="E18" s="51" t="inlineStr">
+      <c r="E18" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2506,17 +3400,17 @@
       <c r="B19" s="22" t="n">
         <v>15</v>
       </c>
-      <c r="C19" s="56" t="inlineStr">
+      <c r="C19" s="58" t="inlineStr">
         <is>
           <t>Workbook opened on a dense tab — not approachable.</t>
         </is>
       </c>
-      <c r="D19" s="56" t="inlineStr">
+      <c r="D19" s="58" t="inlineStr">
         <is>
           <t>Added a clean Home screen (scenario picker + live KPI cards + guided navigation); simple-first tab order.</t>
         </is>
       </c>
-      <c r="E19" s="51" t="inlineStr">
+      <c r="E19" s="53" t="inlineStr">
         <is>
           <t>Resolved</t>
         </is>
@@ -2536,14 +3430,14 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <tabColor rgb="00808A99"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B2:G30"/>
+  <dimension ref="B2:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2563,7 +3457,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="B3" s="57" t="inlineStr">
+      <c r="B3" s="59" t="inlineStr">
         <is>
           <t>Sparkling Daily — One-Year Operating Model</t>
         </is>
@@ -2614,27 +3508,27 @@
       </c>
     </row>
     <row r="7" ht="26" customHeight="1">
-      <c r="B7" s="58">
+      <c r="B7" s="60">
         <f>'Base'!I18</f>
         <v/>
       </c>
-      <c r="C7" s="59">
+      <c r="C7" s="61">
         <f>'Base'!I23</f>
         <v/>
       </c>
-      <c r="D7" s="58">
+      <c r="D7" s="60">
         <f>'Base'!I34</f>
         <v/>
       </c>
-      <c r="E7" s="58">
+      <c r="E7" s="60">
         <f>'Base'!I41</f>
         <v/>
       </c>
-      <c r="F7" s="60">
+      <c r="F7" s="62">
         <f>'Base'!I8</f>
         <v/>
       </c>
-      <c r="G7" s="60">
+      <c r="G7" s="62">
         <f>'Sensitivity'!$C$23</f>
         <v/>
       </c>
@@ -2741,7 +3635,7 @@
           <t>TAB INDEX</t>
         </is>
       </c>
-      <c r="C18" s="61" t="inlineStr"/>
+      <c r="C18" s="63" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="B19" s="24" t="inlineStr">
@@ -2818,54 +3712,90 @@
     <row r="25">
       <c r="B25" s="24" t="inlineStr">
         <is>
-          <t>Sensitivity</t>
+          <t>Pricing Lab</t>
         </is>
       </c>
       <c r="C25" s="21" t="inlineStr">
         <is>
-          <t>Two-way EBITDA table + break-even volume</t>
+          <t>Best wholesale price (CP) per SKU</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="B26" s="24" t="inlineStr">
         <is>
+          <t>Unit Economics</t>
+        </is>
+      </c>
+      <c r="C26" s="21" t="inlineStr">
+        <is>
+          <t>Per-unit costs + suggested retail shelf price</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t>Targets</t>
+        </is>
+      </c>
+      <c r="C27" s="21" t="inlineStr">
+        <is>
+          <t>Goal-seek: price/volume to hit a GP% or EBITDA</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="24" t="inlineStr">
+        <is>
+          <t>Sensitivity</t>
+        </is>
+      </c>
+      <c r="C28" s="21" t="inlineStr">
+        <is>
+          <t>Two-way EBITDA table + break-even volume</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="24" t="inlineStr">
+        <is>
           <t>Checks</t>
         </is>
       </c>
-      <c r="C26" s="21" t="inlineStr">
+      <c r="C29" s="21" t="inlineStr">
         <is>
           <t>Automated validation (should read ALL PASS)</t>
         </is>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="19" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="19" t="inlineStr">
         <is>
           <t>LEGEND</t>
         </is>
       </c>
-      <c r="C28" s="61" t="inlineStr"/>
-    </row>
-    <row r="29">
-      <c r="B29" s="44" t="inlineStr">
+      <c r="C31" s="63" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="B32" s="44" t="inlineStr">
         <is>
           <t>Yellow cell</t>
         </is>
       </c>
-      <c r="C29" s="21" t="inlineStr">
+      <c r="C32" s="21" t="inlineStr">
         <is>
           <t>Input — safe to edit</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="B30" s="62" t="inlineStr">
+    <row r="33">
+      <c r="B33" s="64" t="inlineStr">
         <is>
           <t>Blue tint</t>
         </is>
       </c>
-      <c r="C30" s="21" t="inlineStr">
+      <c r="C33" s="21" t="inlineStr">
         <is>
           <t>Calculated total — do not overwrite</t>
         </is>
@@ -2892,7 +3822,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:O50"/>
+  <dimension ref="B1:O53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -3647,246 +4577,276 @@
         <v>0</v>
       </c>
     </row>
+    <row r="40">
+      <c r="B40" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   3-yr volume growth / yr</t>
+        </is>
+      </c>
+      <c r="C40" s="26" t="n">
+        <v>0.25</v>
+      </c>
+    </row>
     <row r="41">
-      <c r="B41" s="19" t="inlineStr">
+      <c r="B41" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   3-yr price growth / yr</t>
+        </is>
+      </c>
+      <c r="C41" s="26" t="n">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="B42" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   3-yr cost inflation / yr</t>
+        </is>
+      </c>
+      <c r="C42" s="26" t="n">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="B44" s="19" t="inlineStr">
         <is>
           <t>SCENARIO LEVERS</t>
         </is>
       </c>
-      <c r="C41" s="20" t="n"/>
-      <c r="D41" s="20" t="n"/>
-      <c r="E41" s="20" t="n"/>
-      <c r="F41" s="20" t="n"/>
-      <c r="G41" s="20" t="n"/>
-      <c r="H41" s="20" t="n"/>
-      <c r="I41" s="20" t="n"/>
-    </row>
-    <row r="42">
-      <c r="B42" s="17" t="inlineStr">
+      <c r="C44" s="20" t="n"/>
+      <c r="D44" s="20" t="n"/>
+      <c r="E44" s="20" t="n"/>
+      <c r="F44" s="20" t="n"/>
+      <c r="G44" s="20" t="n"/>
+      <c r="H44" s="20" t="n"/>
+      <c r="I44" s="20" t="n"/>
+    </row>
+    <row r="45">
+      <c r="B45" s="17" t="inlineStr">
         <is>
           <t xml:space="preserve">   Scenario</t>
         </is>
       </c>
-      <c r="C42" s="18" t="inlineStr">
+      <c r="C45" s="18" t="inlineStr">
         <is>
           <t>Volume x</t>
         </is>
       </c>
-      <c r="D42" s="18" t="inlineStr">
+      <c r="D45" s="18" t="inlineStr">
         <is>
           <t>Price x</t>
         </is>
       </c>
-      <c r="E42" s="18" t="inlineStr">
+      <c r="E45" s="18" t="inlineStr">
         <is>
           <t>Trade disc Δ</t>
         </is>
-      </c>
-    </row>
-    <row r="43">
-      <c r="B43" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Low</t>
-        </is>
-      </c>
-      <c r="C43" s="32" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="D43" s="32" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="E43" s="26" t="n">
-        <v>0.01</v>
-      </c>
-    </row>
-    <row r="44">
-      <c r="B44" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Base</t>
-        </is>
-      </c>
-      <c r="C44" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="D44" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="E44" s="26" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="45">
-      <c r="B45" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   High</t>
-        </is>
-      </c>
-      <c r="C45" s="32" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="D45" s="32" t="n">
-        <v>1</v>
-      </c>
-      <c r="E45" s="26" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="46">
       <c r="B46" s="31" t="inlineStr">
         <is>
+          <t xml:space="preserve">   Low</t>
+        </is>
+      </c>
+      <c r="C46" s="32" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="D46" s="32" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="E46" s="26" t="n">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="B47" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Base</t>
+        </is>
+      </c>
+      <c r="C47" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="D47" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E47" s="26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="B48" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   High</t>
+        </is>
+      </c>
+      <c r="C48" s="32" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="D48" s="32" t="n">
+        <v>1</v>
+      </c>
+      <c r="E48" s="26" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="B49" s="31" t="inlineStr">
+        <is>
           <t xml:space="preserve">   Stretch</t>
         </is>
       </c>
-      <c r="C46" s="32" t="n">
+      <c r="C49" s="32" t="n">
         <v>1.6</v>
       </c>
-      <c r="D46" s="32" t="n">
+      <c r="D49" s="32" t="n">
         <v>1.05</v>
       </c>
-      <c r="E46" s="26" t="n">
+      <c r="E49" s="26" t="n">
         <v>-0.01</v>
       </c>
     </row>
-    <row r="48">
-      <c r="B48" s="19" t="inlineStr">
+    <row r="51">
+      <c r="B51" s="19" t="inlineStr">
         <is>
           <t>SEASONALITY (% of annual volume)</t>
         </is>
       </c>
-      <c r="C48" s="20" t="n"/>
-      <c r="D48" s="20" t="n"/>
-      <c r="E48" s="20" t="n"/>
-      <c r="F48" s="20" t="n"/>
-      <c r="G48" s="20" t="n"/>
-      <c r="H48" s="20" t="n"/>
-      <c r="I48" s="20" t="n"/>
-      <c r="J48" s="20" t="n"/>
-      <c r="K48" s="20" t="n"/>
-      <c r="L48" s="20" t="n"/>
-      <c r="M48" s="20" t="n"/>
-      <c r="N48" s="20" t="n"/>
-    </row>
-    <row r="49">
-      <c r="C49" s="18" t="inlineStr">
+      <c r="C51" s="20" t="n"/>
+      <c r="D51" s="20" t="n"/>
+      <c r="E51" s="20" t="n"/>
+      <c r="F51" s="20" t="n"/>
+      <c r="G51" s="20" t="n"/>
+      <c r="H51" s="20" t="n"/>
+      <c r="I51" s="20" t="n"/>
+      <c r="J51" s="20" t="n"/>
+      <c r="K51" s="20" t="n"/>
+      <c r="L51" s="20" t="n"/>
+      <c r="M51" s="20" t="n"/>
+      <c r="N51" s="20" t="n"/>
+    </row>
+    <row r="52">
+      <c r="C52" s="18" t="inlineStr">
         <is>
           <t>Jan</t>
         </is>
       </c>
-      <c r="D49" s="18" t="inlineStr">
+      <c r="D52" s="18" t="inlineStr">
         <is>
           <t>Feb</t>
         </is>
       </c>
-      <c r="E49" s="18" t="inlineStr">
+      <c r="E52" s="18" t="inlineStr">
         <is>
           <t>Mar</t>
         </is>
       </c>
-      <c r="F49" s="18" t="inlineStr">
+      <c r="F52" s="18" t="inlineStr">
         <is>
           <t>Apr</t>
         </is>
       </c>
-      <c r="G49" s="18" t="inlineStr">
+      <c r="G52" s="18" t="inlineStr">
         <is>
           <t>May</t>
         </is>
       </c>
-      <c r="H49" s="18" t="inlineStr">
+      <c r="H52" s="18" t="inlineStr">
         <is>
           <t>Jun</t>
         </is>
       </c>
-      <c r="I49" s="18" t="inlineStr">
+      <c r="I52" s="18" t="inlineStr">
         <is>
           <t>Jul</t>
         </is>
       </c>
-      <c r="J49" s="18" t="inlineStr">
+      <c r="J52" s="18" t="inlineStr">
         <is>
           <t>Aug</t>
         </is>
       </c>
-      <c r="K49" s="18" t="inlineStr">
+      <c r="K52" s="18" t="inlineStr">
         <is>
           <t>Sep</t>
         </is>
       </c>
-      <c r="L49" s="18" t="inlineStr">
+      <c r="L52" s="18" t="inlineStr">
         <is>
           <t>Oct</t>
         </is>
       </c>
-      <c r="M49" s="18" t="inlineStr">
+      <c r="M52" s="18" t="inlineStr">
         <is>
           <t>Nov</t>
         </is>
       </c>
-      <c r="N49" s="18" t="inlineStr">
+      <c r="N52" s="18" t="inlineStr">
         <is>
           <t>Dec</t>
         </is>
       </c>
-      <c r="O49" s="18" t="inlineStr">
+      <c r="O52" s="18" t="inlineStr">
         <is>
           <t>Check</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="C50" s="26" t="n">
+    <row r="53">
+      <c r="C53" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="D50" s="26" t="n">
+      <c r="D53" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="E50" s="26" t="n">
+      <c r="E53" s="26" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="F50" s="26" t="n">
+      <c r="F53" s="26" t="n">
         <v>0.08</v>
       </c>
-      <c r="G50" s="26" t="n">
+      <c r="G53" s="26" t="n">
         <v>0.1</v>
       </c>
-      <c r="H50" s="26" t="n">
+      <c r="H53" s="26" t="n">
         <v>0.11</v>
       </c>
-      <c r="I50" s="26" t="n">
+      <c r="I53" s="26" t="n">
         <v>0.12</v>
       </c>
-      <c r="J50" s="26" t="n">
+      <c r="J53" s="26" t="n">
         <v>0.11</v>
       </c>
-      <c r="K50" s="26" t="n">
+      <c r="K53" s="26" t="n">
         <v>0.09</v>
       </c>
-      <c r="L50" s="26" t="n">
+      <c r="L53" s="26" t="n">
         <v>0.08</v>
       </c>
-      <c r="M50" s="26" t="n">
+      <c r="M53" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="N50" s="26" t="n">
+      <c r="N53" s="26" t="n">
         <v>0.06</v>
       </c>
-      <c r="O50" s="33">
-        <f>SUM(C50:N50)</f>
+      <c r="O53" s="33">
+        <f>SUM(C53:N53)</f>
         <v/>
       </c>
     </row>
   </sheetData>
   <mergeCells count="10">
     <mergeCell ref="B30:I30"/>
+    <mergeCell ref="B44:I44"/>
     <mergeCell ref="B6:I6"/>
     <mergeCell ref="B10:I10"/>
     <mergeCell ref="C4:E4"/>
     <mergeCell ref="F4:H4"/>
     <mergeCell ref="B14:I14"/>
     <mergeCell ref="B22:I22"/>
-    <mergeCell ref="B41:I41"/>
-    <mergeCell ref="B48:N48"/>
     <mergeCell ref="B27:I27"/>
+    <mergeCell ref="B51:N51"/>
   </mergeCells>
   <pageMargins left="0.4" right="0.4" top="0.6" bottom="0.6" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" fitToHeight="0" fitToWidth="1"/>
@@ -4460,27 +5420,27 @@
         </is>
       </c>
       <c r="C8" s="36">
-        <f>'Assumptions'!C28*'Assumptions'!$C$44*('Assumptions'!$D$44^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!C28*'Assumptions'!$C$47*('Assumptions'!$D$47^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="D8" s="36">
-        <f>'Assumptions'!D28*'Assumptions'!$C$44*('Assumptions'!$D$44^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!D28*'Assumptions'!$C$47*('Assumptions'!$D$47^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="E8" s="36">
-        <f>'Assumptions'!E28*'Assumptions'!$C$44*('Assumptions'!$D$44^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!E28*'Assumptions'!$C$47*('Assumptions'!$D$47^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="F8" s="36">
-        <f>'Assumptions'!F28*'Assumptions'!$C$44*('Assumptions'!$D$44^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!F28*'Assumptions'!$C$47*('Assumptions'!$D$47^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="G8" s="36">
-        <f>'Assumptions'!G28*'Assumptions'!$C$44*('Assumptions'!$D$44^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!G28*'Assumptions'!$C$47*('Assumptions'!$D$47^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="H8" s="36">
-        <f>'Assumptions'!H28*'Assumptions'!$C$44*('Assumptions'!$D$44^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!H28*'Assumptions'!$C$47*('Assumptions'!$D$47^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="I8" s="42">
@@ -4509,27 +5469,27 @@
         </is>
       </c>
       <c r="C10" s="27">
-        <f>'Assumptions'!C11*'Assumptions'!$D$44</f>
+        <f>'Assumptions'!C11*'Assumptions'!$D$47</f>
         <v/>
       </c>
       <c r="D10" s="27">
-        <f>'Assumptions'!D11*'Assumptions'!$D$44</f>
+        <f>'Assumptions'!D11*'Assumptions'!$D$47</f>
         <v/>
       </c>
       <c r="E10" s="27">
-        <f>'Assumptions'!E11*'Assumptions'!$D$44</f>
+        <f>'Assumptions'!E11*'Assumptions'!$D$47</f>
         <v/>
       </c>
       <c r="F10" s="27">
-        <f>'Assumptions'!F11*'Assumptions'!$D$44</f>
+        <f>'Assumptions'!F11*'Assumptions'!$D$47</f>
         <v/>
       </c>
       <c r="G10" s="27">
-        <f>'Assumptions'!G11*'Assumptions'!$D$44</f>
+        <f>'Assumptions'!G11*'Assumptions'!$D$47</f>
         <v/>
       </c>
       <c r="H10" s="27">
-        <f>'Assumptions'!H11*'Assumptions'!$D$44</f>
+        <f>'Assumptions'!H11*'Assumptions'!$D$47</f>
         <v/>
       </c>
       <c r="I10" s="28">
@@ -4544,27 +5504,27 @@
         </is>
       </c>
       <c r="C11" s="40">
-        <f>'Assumptions'!C12+'Assumptions'!$E$44</f>
+        <f>'Assumptions'!C12+'Assumptions'!$E$47</f>
         <v/>
       </c>
       <c r="D11" s="40">
-        <f>'Assumptions'!D12+'Assumptions'!$E$44</f>
+        <f>'Assumptions'!D12+'Assumptions'!$E$47</f>
         <v/>
       </c>
       <c r="E11" s="40">
-        <f>'Assumptions'!E12+'Assumptions'!$E$44</f>
+        <f>'Assumptions'!E12+'Assumptions'!$E$47</f>
         <v/>
       </c>
       <c r="F11" s="40">
-        <f>'Assumptions'!F12+'Assumptions'!$E$44</f>
+        <f>'Assumptions'!F12+'Assumptions'!$E$47</f>
         <v/>
       </c>
       <c r="G11" s="40">
-        <f>'Assumptions'!G12+'Assumptions'!$E$44</f>
+        <f>'Assumptions'!G12+'Assumptions'!$E$47</f>
         <v/>
       </c>
       <c r="H11" s="40">
-        <f>'Assumptions'!H12+'Assumptions'!$E$44</f>
+        <f>'Assumptions'!H12+'Assumptions'!$E$47</f>
         <v/>
       </c>
       <c r="I11" s="33">
@@ -5481,27 +6441,27 @@
         </is>
       </c>
       <c r="C8" s="36">
-        <f>'Assumptions'!C28*'Assumptions'!$C$43*('Assumptions'!$D$43^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!C28*'Assumptions'!$C$46*('Assumptions'!$D$46^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="D8" s="36">
-        <f>'Assumptions'!D28*'Assumptions'!$C$43*('Assumptions'!$D$43^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!D28*'Assumptions'!$C$46*('Assumptions'!$D$46^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="E8" s="36">
-        <f>'Assumptions'!E28*'Assumptions'!$C$43*('Assumptions'!$D$43^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!E28*'Assumptions'!$C$46*('Assumptions'!$D$46^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="F8" s="36">
-        <f>'Assumptions'!F28*'Assumptions'!$C$43*('Assumptions'!$D$43^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!F28*'Assumptions'!$C$46*('Assumptions'!$D$46^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="G8" s="36">
-        <f>'Assumptions'!G28*'Assumptions'!$C$43*('Assumptions'!$D$43^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!G28*'Assumptions'!$C$46*('Assumptions'!$D$46^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="H8" s="36">
-        <f>'Assumptions'!H28*'Assumptions'!$C$43*('Assumptions'!$D$43^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!H28*'Assumptions'!$C$46*('Assumptions'!$D$46^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="I8" s="42">
@@ -5530,27 +6490,27 @@
         </is>
       </c>
       <c r="C10" s="27">
-        <f>'Assumptions'!C11*'Assumptions'!$D$43</f>
+        <f>'Assumptions'!C11*'Assumptions'!$D$46</f>
         <v/>
       </c>
       <c r="D10" s="27">
-        <f>'Assumptions'!D11*'Assumptions'!$D$43</f>
+        <f>'Assumptions'!D11*'Assumptions'!$D$46</f>
         <v/>
       </c>
       <c r="E10" s="27">
-        <f>'Assumptions'!E11*'Assumptions'!$D$43</f>
+        <f>'Assumptions'!E11*'Assumptions'!$D$46</f>
         <v/>
       </c>
       <c r="F10" s="27">
-        <f>'Assumptions'!F11*'Assumptions'!$D$43</f>
+        <f>'Assumptions'!F11*'Assumptions'!$D$46</f>
         <v/>
       </c>
       <c r="G10" s="27">
-        <f>'Assumptions'!G11*'Assumptions'!$D$43</f>
+        <f>'Assumptions'!G11*'Assumptions'!$D$46</f>
         <v/>
       </c>
       <c r="H10" s="27">
-        <f>'Assumptions'!H11*'Assumptions'!$D$43</f>
+        <f>'Assumptions'!H11*'Assumptions'!$D$46</f>
         <v/>
       </c>
       <c r="I10" s="28">
@@ -5565,27 +6525,27 @@
         </is>
       </c>
       <c r="C11" s="40">
-        <f>'Assumptions'!C12+'Assumptions'!$E$43</f>
+        <f>'Assumptions'!C12+'Assumptions'!$E$46</f>
         <v/>
       </c>
       <c r="D11" s="40">
-        <f>'Assumptions'!D12+'Assumptions'!$E$43</f>
+        <f>'Assumptions'!D12+'Assumptions'!$E$46</f>
         <v/>
       </c>
       <c r="E11" s="40">
-        <f>'Assumptions'!E12+'Assumptions'!$E$43</f>
+        <f>'Assumptions'!E12+'Assumptions'!$E$46</f>
         <v/>
       </c>
       <c r="F11" s="40">
-        <f>'Assumptions'!F12+'Assumptions'!$E$43</f>
+        <f>'Assumptions'!F12+'Assumptions'!$E$46</f>
         <v/>
       </c>
       <c r="G11" s="40">
-        <f>'Assumptions'!G12+'Assumptions'!$E$43</f>
+        <f>'Assumptions'!G12+'Assumptions'!$E$46</f>
         <v/>
       </c>
       <c r="H11" s="40">
-        <f>'Assumptions'!H12+'Assumptions'!$E$43</f>
+        <f>'Assumptions'!H12+'Assumptions'!$E$46</f>
         <v/>
       </c>
       <c r="I11" s="33">
@@ -6502,27 +7462,27 @@
         </is>
       </c>
       <c r="C8" s="36">
-        <f>'Assumptions'!C28*'Assumptions'!$C$45*('Assumptions'!$D$45^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!C28*'Assumptions'!$C$48*('Assumptions'!$D$48^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="D8" s="36">
-        <f>'Assumptions'!D28*'Assumptions'!$C$45*('Assumptions'!$D$45^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!D28*'Assumptions'!$C$48*('Assumptions'!$D$48^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="E8" s="36">
-        <f>'Assumptions'!E28*'Assumptions'!$C$45*('Assumptions'!$D$45^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!E28*'Assumptions'!$C$48*('Assumptions'!$D$48^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="F8" s="36">
-        <f>'Assumptions'!F28*'Assumptions'!$C$45*('Assumptions'!$D$45^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!F28*'Assumptions'!$C$48*('Assumptions'!$D$48^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="G8" s="36">
-        <f>'Assumptions'!G28*'Assumptions'!$C$45*('Assumptions'!$D$45^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!G28*'Assumptions'!$C$48*('Assumptions'!$D$48^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="H8" s="36">
-        <f>'Assumptions'!H28*'Assumptions'!$C$45*('Assumptions'!$D$45^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!H28*'Assumptions'!$C$48*('Assumptions'!$D$48^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="I8" s="42">
@@ -6551,27 +7511,27 @@
         </is>
       </c>
       <c r="C10" s="27">
-        <f>'Assumptions'!C11*'Assumptions'!$D$45</f>
+        <f>'Assumptions'!C11*'Assumptions'!$D$48</f>
         <v/>
       </c>
       <c r="D10" s="27">
-        <f>'Assumptions'!D11*'Assumptions'!$D$45</f>
+        <f>'Assumptions'!D11*'Assumptions'!$D$48</f>
         <v/>
       </c>
       <c r="E10" s="27">
-        <f>'Assumptions'!E11*'Assumptions'!$D$45</f>
+        <f>'Assumptions'!E11*'Assumptions'!$D$48</f>
         <v/>
       </c>
       <c r="F10" s="27">
-        <f>'Assumptions'!F11*'Assumptions'!$D$45</f>
+        <f>'Assumptions'!F11*'Assumptions'!$D$48</f>
         <v/>
       </c>
       <c r="G10" s="27">
-        <f>'Assumptions'!G11*'Assumptions'!$D$45</f>
+        <f>'Assumptions'!G11*'Assumptions'!$D$48</f>
         <v/>
       </c>
       <c r="H10" s="27">
-        <f>'Assumptions'!H11*'Assumptions'!$D$45</f>
+        <f>'Assumptions'!H11*'Assumptions'!$D$48</f>
         <v/>
       </c>
       <c r="I10" s="28">
@@ -6586,27 +7546,27 @@
         </is>
       </c>
       <c r="C11" s="40">
-        <f>'Assumptions'!C12+'Assumptions'!$E$45</f>
+        <f>'Assumptions'!C12+'Assumptions'!$E$48</f>
         <v/>
       </c>
       <c r="D11" s="40">
-        <f>'Assumptions'!D12+'Assumptions'!$E$45</f>
+        <f>'Assumptions'!D12+'Assumptions'!$E$48</f>
         <v/>
       </c>
       <c r="E11" s="40">
-        <f>'Assumptions'!E12+'Assumptions'!$E$45</f>
+        <f>'Assumptions'!E12+'Assumptions'!$E$48</f>
         <v/>
       </c>
       <c r="F11" s="40">
-        <f>'Assumptions'!F12+'Assumptions'!$E$45</f>
+        <f>'Assumptions'!F12+'Assumptions'!$E$48</f>
         <v/>
       </c>
       <c r="G11" s="40">
-        <f>'Assumptions'!G12+'Assumptions'!$E$45</f>
+        <f>'Assumptions'!G12+'Assumptions'!$E$48</f>
         <v/>
       </c>
       <c r="H11" s="40">
-        <f>'Assumptions'!H12+'Assumptions'!$E$45</f>
+        <f>'Assumptions'!H12+'Assumptions'!$E$48</f>
         <v/>
       </c>
       <c r="I11" s="33">
@@ -7523,27 +8483,27 @@
         </is>
       </c>
       <c r="C8" s="36">
-        <f>'Assumptions'!C28*'Assumptions'!$C$46*('Assumptions'!$D$46^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!C28*'Assumptions'!$C$49*('Assumptions'!$D$49^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="D8" s="36">
-        <f>'Assumptions'!D28*'Assumptions'!$C$46*('Assumptions'!$D$46^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!D28*'Assumptions'!$C$49*('Assumptions'!$D$49^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="E8" s="36">
-        <f>'Assumptions'!E28*'Assumptions'!$C$46*('Assumptions'!$D$46^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!E28*'Assumptions'!$C$49*('Assumptions'!$D$49^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="F8" s="36">
-        <f>'Assumptions'!F28*'Assumptions'!$C$46*('Assumptions'!$D$46^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!F28*'Assumptions'!$C$49*('Assumptions'!$D$49^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="G8" s="36">
-        <f>'Assumptions'!G28*'Assumptions'!$C$46*('Assumptions'!$D$46^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!G28*'Assumptions'!$C$49*('Assumptions'!$D$49^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="H8" s="36">
-        <f>'Assumptions'!H28*'Assumptions'!$C$46*('Assumptions'!$D$46^'Assumptions'!$C$39)</f>
+        <f>'Assumptions'!H28*'Assumptions'!$C$49*('Assumptions'!$D$49^'Assumptions'!$C$39)</f>
         <v/>
       </c>
       <c r="I8" s="42">
@@ -7572,27 +8532,27 @@
         </is>
       </c>
       <c r="C10" s="27">
-        <f>'Assumptions'!C11*'Assumptions'!$D$46</f>
+        <f>'Assumptions'!C11*'Assumptions'!$D$49</f>
         <v/>
       </c>
       <c r="D10" s="27">
-        <f>'Assumptions'!D11*'Assumptions'!$D$46</f>
+        <f>'Assumptions'!D11*'Assumptions'!$D$49</f>
         <v/>
       </c>
       <c r="E10" s="27">
-        <f>'Assumptions'!E11*'Assumptions'!$D$46</f>
+        <f>'Assumptions'!E11*'Assumptions'!$D$49</f>
         <v/>
       </c>
       <c r="F10" s="27">
-        <f>'Assumptions'!F11*'Assumptions'!$D$46</f>
+        <f>'Assumptions'!F11*'Assumptions'!$D$49</f>
         <v/>
       </c>
       <c r="G10" s="27">
-        <f>'Assumptions'!G11*'Assumptions'!$D$46</f>
+        <f>'Assumptions'!G11*'Assumptions'!$D$49</f>
         <v/>
       </c>
       <c r="H10" s="27">
-        <f>'Assumptions'!H11*'Assumptions'!$D$46</f>
+        <f>'Assumptions'!H11*'Assumptions'!$D$49</f>
         <v/>
       </c>
       <c r="I10" s="28">
@@ -7607,27 +8567,27 @@
         </is>
       </c>
       <c r="C11" s="40">
-        <f>'Assumptions'!C12+'Assumptions'!$E$46</f>
+        <f>'Assumptions'!C12+'Assumptions'!$E$49</f>
         <v/>
       </c>
       <c r="D11" s="40">
-        <f>'Assumptions'!D12+'Assumptions'!$E$46</f>
+        <f>'Assumptions'!D12+'Assumptions'!$E$49</f>
         <v/>
       </c>
       <c r="E11" s="40">
-        <f>'Assumptions'!E12+'Assumptions'!$E$46</f>
+        <f>'Assumptions'!E12+'Assumptions'!$E$49</f>
         <v/>
       </c>
       <c r="F11" s="40">
-        <f>'Assumptions'!F12+'Assumptions'!$E$46</f>
+        <f>'Assumptions'!F12+'Assumptions'!$E$49</f>
         <v/>
       </c>
       <c r="G11" s="40">
-        <f>'Assumptions'!G12+'Assumptions'!$E$46</f>
+        <f>'Assumptions'!G12+'Assumptions'!$E$49</f>
         <v/>
       </c>
       <c r="H11" s="40">
-        <f>'Assumptions'!H12+'Assumptions'!$E$46</f>
+        <f>'Assumptions'!H12+'Assumptions'!$E$49</f>
         <v/>
       </c>
       <c r="I11" s="33">
@@ -8563,51 +9523,51 @@
         </is>
       </c>
       <c r="C7" s="35">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!C$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!C$53</f>
         <v/>
       </c>
       <c r="D7" s="35">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!D$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!D$53</f>
         <v/>
       </c>
       <c r="E7" s="35">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!E$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!E$53</f>
         <v/>
       </c>
       <c r="F7" s="35">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!F$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!F$53</f>
         <v/>
       </c>
       <c r="G7" s="35">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!G$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!G$53</f>
         <v/>
       </c>
       <c r="H7" s="35">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!H$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!H$53</f>
         <v/>
       </c>
       <c r="I7" s="35">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!I$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!I$53</f>
         <v/>
       </c>
       <c r="J7" s="35">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!J$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!J$53</f>
         <v/>
       </c>
       <c r="K7" s="35">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!K$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!K$53</f>
         <v/>
       </c>
       <c r="L7" s="35">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!L$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!L$53</f>
         <v/>
       </c>
       <c r="M7" s="35">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!M$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!M$53</f>
         <v/>
       </c>
       <c r="N7" s="35">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!N$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I8")*'Assumptions'!N$53</f>
         <v/>
       </c>
       <c r="O7" s="42">
@@ -8622,51 +9582,51 @@
         </is>
       </c>
       <c r="C8" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!C$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!C$53</f>
         <v/>
       </c>
       <c r="D8" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!D$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!D$53</f>
         <v/>
       </c>
       <c r="E8" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!E$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!E$53</f>
         <v/>
       </c>
       <c r="F8" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!F$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!F$53</f>
         <v/>
       </c>
       <c r="G8" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!G$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!G$53</f>
         <v/>
       </c>
       <c r="H8" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!H$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!H$53</f>
         <v/>
       </c>
       <c r="I8" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!I$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!I$53</f>
         <v/>
       </c>
       <c r="J8" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!J$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!J$53</f>
         <v/>
       </c>
       <c r="K8" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!K$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!K$53</f>
         <v/>
       </c>
       <c r="L8" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!L$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!L$53</f>
         <v/>
       </c>
       <c r="M8" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!M$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!M$53</f>
         <v/>
       </c>
       <c r="N8" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!N$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I18")*'Assumptions'!N$53</f>
         <v/>
       </c>
       <c r="O8" s="43">
@@ -8681,51 +9641,51 @@
         </is>
       </c>
       <c r="C9" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!C$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!C$53</f>
         <v/>
       </c>
       <c r="D9" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!D$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!D$53</f>
         <v/>
       </c>
       <c r="E9" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!E$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!E$53</f>
         <v/>
       </c>
       <c r="F9" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!F$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!F$53</f>
         <v/>
       </c>
       <c r="G9" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!G$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!G$53</f>
         <v/>
       </c>
       <c r="H9" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!H$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!H$53</f>
         <v/>
       </c>
       <c r="I9" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!I$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!I$53</f>
         <v/>
       </c>
       <c r="J9" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!J$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!J$53</f>
         <v/>
       </c>
       <c r="K9" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!K$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!K$53</f>
         <v/>
       </c>
       <c r="L9" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!L$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!L$53</f>
         <v/>
       </c>
       <c r="M9" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!M$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!M$53</f>
         <v/>
       </c>
       <c r="N9" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!N$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I22")*'Assumptions'!N$53</f>
         <v/>
       </c>
       <c r="O9" s="43">
@@ -8740,51 +9700,51 @@
         </is>
       </c>
       <c r="C10" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!C$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!C$53</f>
         <v/>
       </c>
       <c r="D10" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!D$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!D$53</f>
         <v/>
       </c>
       <c r="E10" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!E$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!E$53</f>
         <v/>
       </c>
       <c r="F10" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!F$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!F$53</f>
         <v/>
       </c>
       <c r="G10" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!G$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!G$53</f>
         <v/>
       </c>
       <c r="H10" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!H$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!H$53</f>
         <v/>
       </c>
       <c r="I10" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!I$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!I$53</f>
         <v/>
       </c>
       <c r="J10" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!J$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!J$53</f>
         <v/>
       </c>
       <c r="K10" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!K$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!K$53</f>
         <v/>
       </c>
       <c r="L10" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!L$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!L$53</f>
         <v/>
       </c>
       <c r="M10" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!M$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!M$53</f>
         <v/>
       </c>
       <c r="N10" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!N$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I24")*'Assumptions'!N$53</f>
         <v/>
       </c>
       <c r="O10" s="43">
@@ -8799,51 +9759,51 @@
         </is>
       </c>
       <c r="C11" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!C$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!C$53</f>
         <v/>
       </c>
       <c r="D11" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!D$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!D$53</f>
         <v/>
       </c>
       <c r="E11" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!E$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!E$53</f>
         <v/>
       </c>
       <c r="F11" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!F$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!F$53</f>
         <v/>
       </c>
       <c r="G11" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!G$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!G$53</f>
         <v/>
       </c>
       <c r="H11" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!H$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!H$53</f>
         <v/>
       </c>
       <c r="I11" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!I$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!I$53</f>
         <v/>
       </c>
       <c r="J11" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!J$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!J$53</f>
         <v/>
       </c>
       <c r="K11" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!K$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!K$53</f>
         <v/>
       </c>
       <c r="L11" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!L$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!L$53</f>
         <v/>
       </c>
       <c r="M11" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!M$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!M$53</f>
         <v/>
       </c>
       <c r="N11" s="37">
-        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!N$50</f>
+        <f>INDIRECT("'"&amp;$C$4&amp;"'!I25")*'Assumptions'!N$53</f>
         <v/>
       </c>
       <c r="O11" s="43">
@@ -9463,556 +10423,516 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
-    <tabColor rgb="006A1B9A"/>
+    <tabColor rgb="0000695C"/>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="B1:K21"/>
+  <dimension ref="B1:F31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="11" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="11" customWidth="1" min="6" max="6"/>
-    <col width="11" customWidth="1" min="7" max="7"/>
-    <col width="11" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="30" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="B1" s="14" t="inlineStr">
         <is>
-          <t>Sparkling Daily - Pricing Lab (FY2026)</t>
+          <t>Sparkling Daily - 3-Year Projection</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="B2" s="15" t="inlineStr">
         <is>
-          <t>How wholesale price (CP) drives margin. Each column flexes every SKU's CP vs its Assumptions base; volume &amp; costs held at base.</t>
+          <t>Grows the base year by the growth rates on Assumptions. Year 1 = base year, unlevered.</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="B4" s="46" t="inlineStr">
-        <is>
-          <t>Gross Profit %  (by SKU, by CP)</t>
-        </is>
+      <c r="B4" s="21" t="inlineStr">
+        <is>
+          <t>Kgr  base net (Σ vol·cp·(1-d))</t>
+        </is>
+      </c>
+      <c r="C4" s="38">
+        <f>SUMPRODUCT('Assumptions'!C28:H28,'Assumptions'!C11:H11,(1-'Assumptions'!C12:H12))</f>
+        <v/>
       </c>
     </row>
     <row r="5">
-      <c r="B5" s="17" t="inlineStr">
-        <is>
-          <t>SKU  \  CP vs base</t>
-        </is>
-      </c>
-      <c r="C5" s="47" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="D5" s="47" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E5" s="47" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F5" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="G5" s="47" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="H5" s="47" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="I5" s="47" t="n">
-        <v>1.15</v>
+      <c r="B5" s="21" t="inlineStr">
+        <is>
+          <t>Kcos  base COGS (Σ vol·COS/case)</t>
+        </is>
+      </c>
+      <c r="C5" s="38">
+        <f>SUMPRODUCT('Assumptions'!C28:H28,'Assumptions'!C21:H21)</f>
+        <v/>
       </c>
     </row>
     <row r="6">
-      <c r="B6" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Pineapple Singles</t>
-        </is>
-      </c>
-      <c r="C6" s="39">
-        <f>IFERROR(1-'Assumptions'!$C$21/('Assumptions'!$C$11*C$5*(1-'Assumptions'!$C$12)),0)</f>
-        <v/>
-      </c>
-      <c r="D6" s="39">
-        <f>IFERROR(1-'Assumptions'!$C$21/('Assumptions'!$C$11*D$5*(1-'Assumptions'!$C$12)),0)</f>
-        <v/>
-      </c>
-      <c r="E6" s="39">
-        <f>IFERROR(1-'Assumptions'!$C$21/('Assumptions'!$C$11*E$5*(1-'Assumptions'!$C$12)),0)</f>
-        <v/>
-      </c>
-      <c r="F6" s="40">
-        <f>IFERROR(1-'Assumptions'!$C$21/('Assumptions'!$C$11*F$5*(1-'Assumptions'!$C$12)),0)</f>
-        <v/>
-      </c>
-      <c r="G6" s="39">
-        <f>IFERROR(1-'Assumptions'!$C$21/('Assumptions'!$C$11*G$5*(1-'Assumptions'!$C$12)),0)</f>
-        <v/>
-      </c>
-      <c r="H6" s="39">
-        <f>IFERROR(1-'Assumptions'!$C$21/('Assumptions'!$C$11*H$5*(1-'Assumptions'!$C$12)),0)</f>
-        <v/>
-      </c>
-      <c r="I6" s="39">
-        <f>IFERROR(1-'Assumptions'!$C$21/('Assumptions'!$C$11*I$5*(1-'Assumptions'!$C$12)),0)</f>
+      <c r="B6" s="21" t="inlineStr">
+        <is>
+          <t>Kap  base A&amp;P (Σ vol·A&amp;P/case)</t>
+        </is>
+      </c>
+      <c r="C6" s="38">
+        <f>SUMPRODUCT('Assumptions'!C28:H28,'Assumptions'!C26:H26)</f>
         <v/>
       </c>
     </row>
     <row r="7">
-      <c r="B7" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Passionfruit Singles</t>
-        </is>
-      </c>
-      <c r="C7" s="39">
-        <f>IFERROR(1-'Assumptions'!$D$21/('Assumptions'!$D$11*C$5*(1-'Assumptions'!$D$12)),0)</f>
-        <v/>
-      </c>
-      <c r="D7" s="39">
-        <f>IFERROR(1-'Assumptions'!$D$21/('Assumptions'!$D$11*D$5*(1-'Assumptions'!$D$12)),0)</f>
-        <v/>
-      </c>
-      <c r="E7" s="39">
-        <f>IFERROR(1-'Assumptions'!$D$21/('Assumptions'!$D$11*E$5*(1-'Assumptions'!$D$12)),0)</f>
-        <v/>
-      </c>
-      <c r="F7" s="40">
-        <f>IFERROR(1-'Assumptions'!$D$21/('Assumptions'!$D$11*F$5*(1-'Assumptions'!$D$12)),0)</f>
-        <v/>
-      </c>
-      <c r="G7" s="39">
-        <f>IFERROR(1-'Assumptions'!$D$21/('Assumptions'!$D$11*G$5*(1-'Assumptions'!$D$12)),0)</f>
-        <v/>
-      </c>
-      <c r="H7" s="39">
-        <f>IFERROR(1-'Assumptions'!$D$21/('Assumptions'!$D$11*H$5*(1-'Assumptions'!$D$12)),0)</f>
-        <v/>
-      </c>
-      <c r="I7" s="39">
-        <f>IFERROR(1-'Assumptions'!$D$21/('Assumptions'!$D$11*I$5*(1-'Assumptions'!$D$12)),0)</f>
+      <c r="B7" s="21" t="inlineStr">
+        <is>
+          <t>Fixed opex</t>
+        </is>
+      </c>
+      <c r="C7" s="38">
+        <f>'Assumptions'!C31+'Assumptions'!C32+'Assumptions'!C33+'Assumptions'!C34</f>
         <v/>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Lime Lemon Singles</t>
-        </is>
-      </c>
-      <c r="C8" s="39">
-        <f>IFERROR(1-'Assumptions'!$E$21/('Assumptions'!$E$11*C$5*(1-'Assumptions'!$E$12)),0)</f>
-        <v/>
-      </c>
-      <c r="D8" s="39">
-        <f>IFERROR(1-'Assumptions'!$E$21/('Assumptions'!$E$11*D$5*(1-'Assumptions'!$E$12)),0)</f>
-        <v/>
-      </c>
-      <c r="E8" s="39">
-        <f>IFERROR(1-'Assumptions'!$E$21/('Assumptions'!$E$11*E$5*(1-'Assumptions'!$E$12)),0)</f>
-        <v/>
-      </c>
-      <c r="F8" s="40">
-        <f>IFERROR(1-'Assumptions'!$E$21/('Assumptions'!$E$11*F$5*(1-'Assumptions'!$E$12)),0)</f>
-        <v/>
-      </c>
-      <c r="G8" s="39">
-        <f>IFERROR(1-'Assumptions'!$E$21/('Assumptions'!$E$11*G$5*(1-'Assumptions'!$E$12)),0)</f>
-        <v/>
-      </c>
-      <c r="H8" s="39">
-        <f>IFERROR(1-'Assumptions'!$E$21/('Assumptions'!$E$11*H$5*(1-'Assumptions'!$E$12)),0)</f>
-        <v/>
-      </c>
-      <c r="I8" s="39">
-        <f>IFERROR(1-'Assumptions'!$E$21/('Assumptions'!$E$11*I$5*(1-'Assumptions'!$E$12)),0)</f>
+      <c r="B8" s="21" t="inlineStr">
+        <is>
+          <t>Logistics % of net</t>
+        </is>
+      </c>
+      <c r="C8" s="40">
+        <f>'Assumptions'!C35</f>
         <v/>
       </c>
     </row>
     <row r="9">
-      <c r="B9" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Pineapple 4-Pack</t>
-        </is>
-      </c>
-      <c r="C9" s="39">
-        <f>IFERROR(1-'Assumptions'!$F$21/('Assumptions'!$F$11*C$5*(1-'Assumptions'!$F$12)),0)</f>
-        <v/>
-      </c>
-      <c r="D9" s="39">
-        <f>IFERROR(1-'Assumptions'!$F$21/('Assumptions'!$F$11*D$5*(1-'Assumptions'!$F$12)),0)</f>
-        <v/>
-      </c>
-      <c r="E9" s="39">
-        <f>IFERROR(1-'Assumptions'!$F$21/('Assumptions'!$F$11*E$5*(1-'Assumptions'!$F$12)),0)</f>
-        <v/>
-      </c>
-      <c r="F9" s="40">
-        <f>IFERROR(1-'Assumptions'!$F$21/('Assumptions'!$F$11*F$5*(1-'Assumptions'!$F$12)),0)</f>
-        <v/>
-      </c>
-      <c r="G9" s="39">
-        <f>IFERROR(1-'Assumptions'!$F$21/('Assumptions'!$F$11*G$5*(1-'Assumptions'!$F$12)),0)</f>
-        <v/>
-      </c>
-      <c r="H9" s="39">
-        <f>IFERROR(1-'Assumptions'!$F$21/('Assumptions'!$F$11*H$5*(1-'Assumptions'!$F$12)),0)</f>
-        <v/>
-      </c>
-      <c r="I9" s="39">
-        <f>IFERROR(1-'Assumptions'!$F$21/('Assumptions'!$F$11*I$5*(1-'Assumptions'!$F$12)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="10">
-      <c r="B10" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Passionfruit 4-Pack</t>
-        </is>
-      </c>
-      <c r="C10" s="39">
-        <f>IFERROR(1-'Assumptions'!$G$21/('Assumptions'!$G$11*C$5*(1-'Assumptions'!$G$12)),0)</f>
-        <v/>
-      </c>
-      <c r="D10" s="39">
-        <f>IFERROR(1-'Assumptions'!$G$21/('Assumptions'!$G$11*D$5*(1-'Assumptions'!$G$12)),0)</f>
-        <v/>
-      </c>
-      <c r="E10" s="39">
-        <f>IFERROR(1-'Assumptions'!$G$21/('Assumptions'!$G$11*E$5*(1-'Assumptions'!$G$12)),0)</f>
-        <v/>
-      </c>
-      <c r="F10" s="40">
-        <f>IFERROR(1-'Assumptions'!$G$21/('Assumptions'!$G$11*F$5*(1-'Assumptions'!$G$12)),0)</f>
-        <v/>
-      </c>
-      <c r="G10" s="39">
-        <f>IFERROR(1-'Assumptions'!$G$21/('Assumptions'!$G$11*G$5*(1-'Assumptions'!$G$12)),0)</f>
-        <v/>
-      </c>
-      <c r="H10" s="39">
-        <f>IFERROR(1-'Assumptions'!$G$21/('Assumptions'!$G$11*H$5*(1-'Assumptions'!$G$12)),0)</f>
-        <v/>
-      </c>
-      <c r="I10" s="39">
-        <f>IFERROR(1-'Assumptions'!$G$21/('Assumptions'!$G$11*I$5*(1-'Assumptions'!$G$12)),0)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="11">
-      <c r="B11" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Lime Lemon 4-Pack</t>
-        </is>
-      </c>
-      <c r="C11" s="39">
-        <f>IFERROR(1-'Assumptions'!$H$21/('Assumptions'!$H$11*C$5*(1-'Assumptions'!$H$12)),0)</f>
-        <v/>
-      </c>
-      <c r="D11" s="39">
-        <f>IFERROR(1-'Assumptions'!$H$21/('Assumptions'!$H$11*D$5*(1-'Assumptions'!$H$12)),0)</f>
-        <v/>
-      </c>
-      <c r="E11" s="39">
-        <f>IFERROR(1-'Assumptions'!$H$21/('Assumptions'!$H$11*E$5*(1-'Assumptions'!$H$12)),0)</f>
-        <v/>
-      </c>
-      <c r="F11" s="40">
-        <f>IFERROR(1-'Assumptions'!$H$21/('Assumptions'!$H$11*F$5*(1-'Assumptions'!$H$12)),0)</f>
-        <v/>
-      </c>
-      <c r="G11" s="39">
-        <f>IFERROR(1-'Assumptions'!$H$21/('Assumptions'!$H$11*G$5*(1-'Assumptions'!$H$12)),0)</f>
-        <v/>
-      </c>
-      <c r="H11" s="39">
-        <f>IFERROR(1-'Assumptions'!$H$21/('Assumptions'!$H$11*H$5*(1-'Assumptions'!$H$12)),0)</f>
-        <v/>
-      </c>
-      <c r="I11" s="39">
-        <f>IFERROR(1-'Assumptions'!$H$21/('Assumptions'!$H$11*I$5*(1-'Assumptions'!$H$12)),0)</f>
+      <c r="B9" s="21" t="inlineStr">
+        <is>
+          <t>Base total cases</t>
+        </is>
+      </c>
+      <c r="C9" s="36">
+        <f>SUM('Assumptions'!C28:H28)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>3-Year (CDN $)</t>
+        </is>
+      </c>
+      <c r="C12" s="18" t="inlineStr">
+        <is>
+          <t>Year 1</t>
+        </is>
+      </c>
+      <c r="D12" s="18" t="inlineStr">
+        <is>
+          <t>Year 2</t>
+        </is>
+      </c>
+      <c r="E12" s="18" t="inlineStr">
+        <is>
+          <t>Year 3</t>
+        </is>
+      </c>
+      <c r="F12" s="18" t="inlineStr">
+        <is>
+          <t>CAGR</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Physical Cases</t>
+        </is>
+      </c>
+      <c r="C13" s="46">
+        <f>(1+'Assumptions'!$C$40)^0*$C$9</f>
+        <v/>
+      </c>
+      <c r="D13" s="46">
+        <f>(1+'Assumptions'!$C$40)^1*$C$9</f>
+        <v/>
+      </c>
+      <c r="E13" s="46">
+        <f>(1+'Assumptions'!$C$40)^2*$C$9</f>
+        <v/>
+      </c>
+      <c r="F13" s="40">
+        <f>IFERROR((E13/C13)^(1/2)-1,"")</f>
         <v/>
       </c>
     </row>
     <row r="14">
-      <c r="B14" s="46" t="inlineStr">
-        <is>
-          <t>Annual Contribution $  (by SKU, by CP — demand-adjusted)</t>
-        </is>
+      <c r="B14" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Net Sales</t>
+        </is>
+      </c>
+      <c r="C14" s="47">
+        <f>(1+'Assumptions'!$C$40)^0*(1+'Assumptions'!$C$41)^0*$C$4</f>
+        <v/>
+      </c>
+      <c r="D14" s="47">
+        <f>(1+'Assumptions'!$C$40)^1*(1+'Assumptions'!$C$41)^1*$C$4</f>
+        <v/>
+      </c>
+      <c r="E14" s="47">
+        <f>(1+'Assumptions'!$C$40)^2*(1+'Assumptions'!$C$41)^2*$C$4</f>
+        <v/>
+      </c>
+      <c r="F14" s="40">
+        <f>IFERROR((E14/C14)^(1/2)-1,"")</f>
+        <v/>
       </c>
     </row>
     <row r="15">
-      <c r="B15" s="17" t="inlineStr">
-        <is>
-          <t>SKU  \  CP vs base</t>
-        </is>
-      </c>
-      <c r="C15" s="47" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="D15" s="47" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="E15" s="47" t="n">
-        <v>0.95</v>
-      </c>
-      <c r="F15" s="47" t="n">
-        <v>1</v>
-      </c>
-      <c r="G15" s="47" t="n">
-        <v>1.05</v>
-      </c>
-      <c r="H15" s="47" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="I15" s="47" t="n">
-        <v>1.15</v>
-      </c>
-      <c r="K15" s="18" t="inlineStr">
-        <is>
-          <t>Best CP ×</t>
-        </is>
+      <c r="B15" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Cost of Sales</t>
+        </is>
+      </c>
+      <c r="C15" s="37">
+        <f>(1+'Assumptions'!$C$40)^0*(1+'Assumptions'!$C$42)^0*$C$5</f>
+        <v/>
+      </c>
+      <c r="D15" s="37">
+        <f>(1+'Assumptions'!$C$40)^1*(1+'Assumptions'!$C$42)^1*$C$5</f>
+        <v/>
+      </c>
+      <c r="E15" s="37">
+        <f>(1+'Assumptions'!$C$40)^2*(1+'Assumptions'!$C$42)^2*$C$5</f>
+        <v/>
+      </c>
+      <c r="F15" s="40">
+        <f>IFERROR((E15/C15)^(1/2)-1,"")</f>
+        <v/>
       </c>
     </row>
     <row r="16">
-      <c r="B16" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Pineapple Singles</t>
-        </is>
-      </c>
-      <c r="C16" s="37">
-        <f>'Assumptions'!$C$28*(C$15^'Assumptions'!$C$39)*(('Assumptions'!$C$11*C$15*(1-'Assumptions'!$C$12))-'Assumptions'!$C$21-'Assumptions'!$C$26)</f>
-        <v/>
-      </c>
-      <c r="D16" s="37">
-        <f>'Assumptions'!$C$28*(D$15^'Assumptions'!$C$39)*(('Assumptions'!$C$11*D$15*(1-'Assumptions'!$C$12))-'Assumptions'!$C$21-'Assumptions'!$C$26)</f>
-        <v/>
-      </c>
-      <c r="E16" s="37">
-        <f>'Assumptions'!$C$28*(E$15^'Assumptions'!$C$39)*(('Assumptions'!$C$11*E$15*(1-'Assumptions'!$C$12))-'Assumptions'!$C$21-'Assumptions'!$C$26)</f>
-        <v/>
-      </c>
-      <c r="F16" s="38">
-        <f>'Assumptions'!$C$28*(F$15^'Assumptions'!$C$39)*(('Assumptions'!$C$11*F$15*(1-'Assumptions'!$C$12))-'Assumptions'!$C$21-'Assumptions'!$C$26)</f>
-        <v/>
-      </c>
-      <c r="G16" s="37">
-        <f>'Assumptions'!$C$28*(G$15^'Assumptions'!$C$39)*(('Assumptions'!$C$11*G$15*(1-'Assumptions'!$C$12))-'Assumptions'!$C$21-'Assumptions'!$C$26)</f>
-        <v/>
-      </c>
-      <c r="H16" s="37">
-        <f>'Assumptions'!$C$28*(H$15^'Assumptions'!$C$39)*(('Assumptions'!$C$11*H$15*(1-'Assumptions'!$C$12))-'Assumptions'!$C$21-'Assumptions'!$C$26)</f>
-        <v/>
-      </c>
-      <c r="I16" s="37">
-        <f>'Assumptions'!$C$28*(I$15^'Assumptions'!$C$39)*(('Assumptions'!$C$11*I$15*(1-'Assumptions'!$C$12))-'Assumptions'!$C$21-'Assumptions'!$C$26)</f>
-        <v/>
-      </c>
-      <c r="K16" s="48">
-        <f>INDEX($C$15:$I$15,MATCH(MAX(C16:I16),C16:I16,0))</f>
+      <c r="B16" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Gross Profit</t>
+        </is>
+      </c>
+      <c r="C16" s="47">
+        <f>C14-C15</f>
+        <v/>
+      </c>
+      <c r="D16" s="47">
+        <f>D14-D15</f>
+        <v/>
+      </c>
+      <c r="E16" s="47">
+        <f>E14-E15</f>
+        <v/>
+      </c>
+      <c r="F16" s="40">
+        <f>IFERROR((E16/C16)^(1/2)-1,"")</f>
         <v/>
       </c>
     </row>
     <row r="17">
-      <c r="B17" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Passionfruit Singles</t>
-        </is>
-      </c>
-      <c r="C17" s="37">
-        <f>'Assumptions'!$D$28*(C$15^'Assumptions'!$C$39)*(('Assumptions'!$D$11*C$15*(1-'Assumptions'!$D$12))-'Assumptions'!$D$21-'Assumptions'!$D$26)</f>
-        <v/>
-      </c>
-      <c r="D17" s="37">
-        <f>'Assumptions'!$D$28*(D$15^'Assumptions'!$C$39)*(('Assumptions'!$D$11*D$15*(1-'Assumptions'!$D$12))-'Assumptions'!$D$21-'Assumptions'!$D$26)</f>
-        <v/>
-      </c>
-      <c r="E17" s="37">
-        <f>'Assumptions'!$D$28*(E$15^'Assumptions'!$C$39)*(('Assumptions'!$D$11*E$15*(1-'Assumptions'!$D$12))-'Assumptions'!$D$21-'Assumptions'!$D$26)</f>
-        <v/>
-      </c>
-      <c r="F17" s="38">
-        <f>'Assumptions'!$D$28*(F$15^'Assumptions'!$C$39)*(('Assumptions'!$D$11*F$15*(1-'Assumptions'!$D$12))-'Assumptions'!$D$21-'Assumptions'!$D$26)</f>
-        <v/>
-      </c>
-      <c r="G17" s="37">
-        <f>'Assumptions'!$D$28*(G$15^'Assumptions'!$C$39)*(('Assumptions'!$D$11*G$15*(1-'Assumptions'!$D$12))-'Assumptions'!$D$21-'Assumptions'!$D$26)</f>
-        <v/>
-      </c>
-      <c r="H17" s="37">
-        <f>'Assumptions'!$D$28*(H$15^'Assumptions'!$C$39)*(('Assumptions'!$D$11*H$15*(1-'Assumptions'!$D$12))-'Assumptions'!$D$21-'Assumptions'!$D$26)</f>
-        <v/>
-      </c>
-      <c r="I17" s="37">
-        <f>'Assumptions'!$D$28*(I$15^'Assumptions'!$C$39)*(('Assumptions'!$D$11*I$15*(1-'Assumptions'!$D$12))-'Assumptions'!$D$21-'Assumptions'!$D$26)</f>
-        <v/>
-      </c>
-      <c r="K17" s="48">
-        <f>INDEX($C$15:$I$15,MATCH(MAX(C17:I17),C17:I17,0))</f>
+      <c r="B17" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   GP %</t>
+        </is>
+      </c>
+      <c r="C17" s="39">
+        <f>IFERROR(C16/C14,0)</f>
+        <v/>
+      </c>
+      <c r="D17" s="39">
+        <f>IFERROR(D16/D14,0)</f>
+        <v/>
+      </c>
+      <c r="E17" s="39">
+        <f>IFERROR(E16/E14,0)</f>
         <v/>
       </c>
     </row>
     <row r="18">
-      <c r="B18" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Lime Lemon Singles</t>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   A&amp;P</t>
         </is>
       </c>
       <c r="C18" s="37">
-        <f>'Assumptions'!$E$28*(C$15^'Assumptions'!$C$39)*(('Assumptions'!$E$11*C$15*(1-'Assumptions'!$E$12))-'Assumptions'!$E$21-'Assumptions'!$E$26)</f>
+        <f>(1+'Assumptions'!$C$40)^0*$C$6</f>
         <v/>
       </c>
       <c r="D18" s="37">
-        <f>'Assumptions'!$E$28*(D$15^'Assumptions'!$C$39)*(('Assumptions'!$E$11*D$15*(1-'Assumptions'!$E$12))-'Assumptions'!$E$21-'Assumptions'!$E$26)</f>
+        <f>(1+'Assumptions'!$C$40)^1*$C$6</f>
         <v/>
       </c>
       <c r="E18" s="37">
-        <f>'Assumptions'!$E$28*(E$15^'Assumptions'!$C$39)*(('Assumptions'!$E$11*E$15*(1-'Assumptions'!$E$12))-'Assumptions'!$E$21-'Assumptions'!$E$26)</f>
-        <v/>
-      </c>
-      <c r="F18" s="38">
-        <f>'Assumptions'!$E$28*(F$15^'Assumptions'!$C$39)*(('Assumptions'!$E$11*F$15*(1-'Assumptions'!$E$12))-'Assumptions'!$E$21-'Assumptions'!$E$26)</f>
-        <v/>
-      </c>
-      <c r="G18" s="37">
-        <f>'Assumptions'!$E$28*(G$15^'Assumptions'!$C$39)*(('Assumptions'!$E$11*G$15*(1-'Assumptions'!$E$12))-'Assumptions'!$E$21-'Assumptions'!$E$26)</f>
-        <v/>
-      </c>
-      <c r="H18" s="37">
-        <f>'Assumptions'!$E$28*(H$15^'Assumptions'!$C$39)*(('Assumptions'!$E$11*H$15*(1-'Assumptions'!$E$12))-'Assumptions'!$E$21-'Assumptions'!$E$26)</f>
-        <v/>
-      </c>
-      <c r="I18" s="37">
-        <f>'Assumptions'!$E$28*(I$15^'Assumptions'!$C$39)*(('Assumptions'!$E$11*I$15*(1-'Assumptions'!$E$12))-'Assumptions'!$E$21-'Assumptions'!$E$26)</f>
-        <v/>
-      </c>
-      <c r="K18" s="48">
-        <f>INDEX($C$15:$I$15,MATCH(MAX(C18:I18),C18:I18,0))</f>
+        <f>(1+'Assumptions'!$C$40)^2*$C$6</f>
+        <v/>
+      </c>
+      <c r="F18" s="40">
+        <f>IFERROR((E18/C18)^(1/2)-1,"")</f>
         <v/>
       </c>
     </row>
     <row r="19">
-      <c r="B19" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Pineapple 4-Pack</t>
-        </is>
-      </c>
-      <c r="C19" s="37">
-        <f>'Assumptions'!$F$28*(C$15^'Assumptions'!$C$39)*(('Assumptions'!$F$11*C$15*(1-'Assumptions'!$F$12))-'Assumptions'!$F$21-'Assumptions'!$F$26)</f>
-        <v/>
-      </c>
-      <c r="D19" s="37">
-        <f>'Assumptions'!$F$28*(D$15^'Assumptions'!$C$39)*(('Assumptions'!$F$11*D$15*(1-'Assumptions'!$F$12))-'Assumptions'!$F$21-'Assumptions'!$F$26)</f>
-        <v/>
-      </c>
-      <c r="E19" s="37">
-        <f>'Assumptions'!$F$28*(E$15^'Assumptions'!$C$39)*(('Assumptions'!$F$11*E$15*(1-'Assumptions'!$F$12))-'Assumptions'!$F$21-'Assumptions'!$F$26)</f>
-        <v/>
-      </c>
-      <c r="F19" s="38">
-        <f>'Assumptions'!$F$28*(F$15^'Assumptions'!$C$39)*(('Assumptions'!$F$11*F$15*(1-'Assumptions'!$F$12))-'Assumptions'!$F$21-'Assumptions'!$F$26)</f>
-        <v/>
-      </c>
-      <c r="G19" s="37">
-        <f>'Assumptions'!$F$28*(G$15^'Assumptions'!$C$39)*(('Assumptions'!$F$11*G$15*(1-'Assumptions'!$F$12))-'Assumptions'!$F$21-'Assumptions'!$F$26)</f>
-        <v/>
-      </c>
-      <c r="H19" s="37">
-        <f>'Assumptions'!$F$28*(H$15^'Assumptions'!$C$39)*(('Assumptions'!$F$11*H$15*(1-'Assumptions'!$F$12))-'Assumptions'!$F$21-'Assumptions'!$F$26)</f>
-        <v/>
-      </c>
-      <c r="I19" s="37">
-        <f>'Assumptions'!$F$28*(I$15^'Assumptions'!$C$39)*(('Assumptions'!$F$11*I$15*(1-'Assumptions'!$F$12))-'Assumptions'!$F$21-'Assumptions'!$F$26)</f>
-        <v/>
-      </c>
-      <c r="K19" s="48">
-        <f>INDEX($C$15:$I$15,MATCH(MAX(C19:I19),C19:I19,0))</f>
+      <c r="B19" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Contribution</t>
+        </is>
+      </c>
+      <c r="C19" s="47">
+        <f>C16-C18</f>
+        <v/>
+      </c>
+      <c r="D19" s="47">
+        <f>D16-D18</f>
+        <v/>
+      </c>
+      <c r="E19" s="47">
+        <f>E16-E18</f>
+        <v/>
+      </c>
+      <c r="F19" s="40">
+        <f>IFERROR((E19/C19)^(1/2)-1,"")</f>
         <v/>
       </c>
     </row>
     <row r="20">
-      <c r="B20" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Passionfruit 4-Pack</t>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Logistics</t>
         </is>
       </c>
       <c r="C20" s="37">
-        <f>'Assumptions'!$G$28*(C$15^'Assumptions'!$C$39)*(('Assumptions'!$G$11*C$15*(1-'Assumptions'!$G$12))-'Assumptions'!$G$21-'Assumptions'!$G$26)</f>
+        <f>$C$8*C14</f>
         <v/>
       </c>
       <c r="D20" s="37">
-        <f>'Assumptions'!$G$28*(D$15^'Assumptions'!$C$39)*(('Assumptions'!$G$11*D$15*(1-'Assumptions'!$G$12))-'Assumptions'!$G$21-'Assumptions'!$G$26)</f>
+        <f>$C$8*D14</f>
         <v/>
       </c>
       <c r="E20" s="37">
-        <f>'Assumptions'!$G$28*(E$15^'Assumptions'!$C$39)*(('Assumptions'!$G$11*E$15*(1-'Assumptions'!$G$12))-'Assumptions'!$G$21-'Assumptions'!$G$26)</f>
-        <v/>
-      </c>
-      <c r="F20" s="38">
-        <f>'Assumptions'!$G$28*(F$15^'Assumptions'!$C$39)*(('Assumptions'!$G$11*F$15*(1-'Assumptions'!$G$12))-'Assumptions'!$G$21-'Assumptions'!$G$26)</f>
-        <v/>
-      </c>
-      <c r="G20" s="37">
-        <f>'Assumptions'!$G$28*(G$15^'Assumptions'!$C$39)*(('Assumptions'!$G$11*G$15*(1-'Assumptions'!$G$12))-'Assumptions'!$G$21-'Assumptions'!$G$26)</f>
-        <v/>
-      </c>
-      <c r="H20" s="37">
-        <f>'Assumptions'!$G$28*(H$15^'Assumptions'!$C$39)*(('Assumptions'!$G$11*H$15*(1-'Assumptions'!$G$12))-'Assumptions'!$G$21-'Assumptions'!$G$26)</f>
-        <v/>
-      </c>
-      <c r="I20" s="37">
-        <f>'Assumptions'!$G$28*(I$15^'Assumptions'!$C$39)*(('Assumptions'!$G$11*I$15*(1-'Assumptions'!$G$12))-'Assumptions'!$G$21-'Assumptions'!$G$26)</f>
-        <v/>
-      </c>
-      <c r="K20" s="48">
-        <f>INDEX($C$15:$I$15,MATCH(MAX(C20:I20),C20:I20,0))</f>
+        <f>$C$8*E14</f>
+        <v/>
+      </c>
+      <c r="F20" s="40">
+        <f>IFERROR((E20/C20)^(1/2)-1,"")</f>
         <v/>
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="34" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   Lime Lemon 4-Pack</t>
+      <c r="B21" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Fixed opex</t>
         </is>
       </c>
       <c r="C21" s="37">
-        <f>'Assumptions'!$H$28*(C$15^'Assumptions'!$C$39)*(('Assumptions'!$H$11*C$15*(1-'Assumptions'!$H$12))-'Assumptions'!$H$21-'Assumptions'!$H$26)</f>
+        <f>$C$7</f>
         <v/>
       </c>
       <c r="D21" s="37">
-        <f>'Assumptions'!$H$28*(D$15^'Assumptions'!$C$39)*(('Assumptions'!$H$11*D$15*(1-'Assumptions'!$H$12))-'Assumptions'!$H$21-'Assumptions'!$H$26)</f>
+        <f>$C$7</f>
         <v/>
       </c>
       <c r="E21" s="37">
-        <f>'Assumptions'!$H$28*(E$15^'Assumptions'!$C$39)*(('Assumptions'!$H$11*E$15*(1-'Assumptions'!$H$12))-'Assumptions'!$H$21-'Assumptions'!$H$26)</f>
-        <v/>
-      </c>
-      <c r="F21" s="38">
-        <f>'Assumptions'!$H$28*(F$15^'Assumptions'!$C$39)*(('Assumptions'!$H$11*F$15*(1-'Assumptions'!$H$12))-'Assumptions'!$H$21-'Assumptions'!$H$26)</f>
-        <v/>
-      </c>
-      <c r="G21" s="37">
-        <f>'Assumptions'!$H$28*(G$15^'Assumptions'!$C$39)*(('Assumptions'!$H$11*G$15*(1-'Assumptions'!$H$12))-'Assumptions'!$H$21-'Assumptions'!$H$26)</f>
-        <v/>
-      </c>
-      <c r="H21" s="37">
-        <f>'Assumptions'!$H$28*(H$15^'Assumptions'!$C$39)*(('Assumptions'!$H$11*H$15*(1-'Assumptions'!$H$12))-'Assumptions'!$H$21-'Assumptions'!$H$26)</f>
-        <v/>
-      </c>
-      <c r="I21" s="37">
-        <f>'Assumptions'!$H$28*(I$15^'Assumptions'!$C$39)*(('Assumptions'!$H$11*I$15*(1-'Assumptions'!$H$12))-'Assumptions'!$H$21-'Assumptions'!$H$26)</f>
-        <v/>
-      </c>
-      <c r="K21" s="48">
-        <f>INDEX($C$15:$I$15,MATCH(MAX(C21:I21),C21:I21,0))</f>
-        <v/>
+        <f>$C$7</f>
+        <v/>
+      </c>
+      <c r="F21" s="40">
+        <f>IFERROR((E21/C21)^(1/2)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   EBITDA</t>
+        </is>
+      </c>
+      <c r="C22" s="47">
+        <f>C19-C20-C21</f>
+        <v/>
+      </c>
+      <c r="D22" s="47">
+        <f>D19-D20-D21</f>
+        <v/>
+      </c>
+      <c r="E22" s="47">
+        <f>E19-E20-E21</f>
+        <v/>
+      </c>
+      <c r="F22" s="40">
+        <f>IFERROR((E22/C22)^(1/2)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   EBITDA %</t>
+        </is>
+      </c>
+      <c r="C23" s="39">
+        <f>IFERROR(C22/C14,0)</f>
+        <v/>
+      </c>
+      <c r="D23" s="39">
+        <f>IFERROR(D22/D14,0)</f>
+        <v/>
+      </c>
+      <c r="E23" s="39">
+        <f>IFERROR(E22/E14,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   D&amp;A</t>
+        </is>
+      </c>
+      <c r="C24" s="37">
+        <f>'Assumptions'!$C$36</f>
+        <v/>
+      </c>
+      <c r="D24" s="37">
+        <f>'Assumptions'!$C$36</f>
+        <v/>
+      </c>
+      <c r="E24" s="37">
+        <f>'Assumptions'!$C$36</f>
+        <v/>
+      </c>
+      <c r="F24" s="40">
+        <f>IFERROR((E24/C24)^(1/2)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   EBIT</t>
+        </is>
+      </c>
+      <c r="C25" s="47">
+        <f>C22-C24</f>
+        <v/>
+      </c>
+      <c r="D25" s="47">
+        <f>D22-D24</f>
+        <v/>
+      </c>
+      <c r="E25" s="47">
+        <f>E22-E24</f>
+        <v/>
+      </c>
+      <c r="F25" s="40">
+        <f>IFERROR((E25/C25)^(1/2)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Interest</t>
+        </is>
+      </c>
+      <c r="C26" s="37">
+        <f>'Assumptions'!$C$37</f>
+        <v/>
+      </c>
+      <c r="D26" s="37">
+        <f>'Assumptions'!$C$37</f>
+        <v/>
+      </c>
+      <c r="E26" s="37">
+        <f>'Assumptions'!$C$37</f>
+        <v/>
+      </c>
+      <c r="F26" s="40">
+        <f>IFERROR((E26/C26)^(1/2)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Pre-tax Profit</t>
+        </is>
+      </c>
+      <c r="C27" s="47">
+        <f>C25-C26</f>
+        <v/>
+      </c>
+      <c r="D27" s="47">
+        <f>D25-D26</f>
+        <v/>
+      </c>
+      <c r="E27" s="47">
+        <f>E25-E26</f>
+        <v/>
+      </c>
+      <c r="F27" s="40">
+        <f>IFERROR((E27/C27)^(1/2)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Tax</t>
+        </is>
+      </c>
+      <c r="C28" s="37">
+        <f>MAX(0,C27*'Assumptions'!$C$38)</f>
+        <v/>
+      </c>
+      <c r="D28" s="37">
+        <f>MAX(0,D27*'Assumptions'!$C$38)</f>
+        <v/>
+      </c>
+      <c r="E28" s="37">
+        <f>MAX(0,E27*'Assumptions'!$C$38)</f>
+        <v/>
+      </c>
+      <c r="F28" s="40">
+        <f>IFERROR((E28/C28)^(1/2)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Net Income</t>
+        </is>
+      </c>
+      <c r="C29" s="47">
+        <f>C27-C28</f>
+        <v/>
+      </c>
+      <c r="D29" s="47">
+        <f>D27-D28</f>
+        <v/>
+      </c>
+      <c r="E29" s="47">
+        <f>E27-E28</f>
+        <v/>
+      </c>
+      <c r="F29" s="40">
+        <f>IFERROR((E29/C29)^(1/2)-1,"")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31">
+      <c r="B31" s="15" t="inlineStr">
+        <is>
+          <t>Year 1 = base year. Years 2-3 compound the growth rates. CAGR = annual growth across the 3 years.</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Correct flavour names to Raspberry, Lime Lemon, Passion Fruit Pineapple
The model listed Pineapple and Passionfruit as two separate flavours and
had no Raspberry. Rename in the HTML app, the workbook builder and the
rebuilt workbook so all three match the real line.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XtU4ZhhiP3B25DcbgYH1Pu
</commit_message>
<xml_diff>
--- a/Organika_Sparkling_Daily_1YR_Scenario_Model.xlsx
+++ b/Organika_Sparkling_Daily_1YR_Scenario_Model.xlsx
@@ -26,7 +26,7 @@
     <sheet name="Cover" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <definedNames>
-    <definedName name="CP_Pineapple_Singles">'Assumptions'!$C$11</definedName>
+    <definedName name="CP_Raspberry_Singles">'Assumptions'!$C$11</definedName>
     <definedName name="BaseVolume_Total">'Assumptions'!$C$28:$H$28</definedName>
     <definedName name="TaxRate">'Assumptions'!$C$38</definedName>
     <definedName name="LogisticsPct">'Assumptions'!$C$35</definedName>
@@ -1136,7 +1136,7 @@
     <row r="6">
       <c r="B6" s="34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Pineapple Singles</t>
+          <t xml:space="preserve">   Raspberry Singles</t>
         </is>
       </c>
       <c r="C6" s="39">
@@ -1171,7 +1171,7 @@
     <row r="7">
       <c r="B7" s="34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Passionfruit Singles</t>
+          <t xml:space="preserve">   Passion Fruit Pineapple Singles</t>
         </is>
       </c>
       <c r="C7" s="39">
@@ -1241,7 +1241,7 @@
     <row r="9">
       <c r="B9" s="34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Pineapple 4-Pack</t>
+          <t xml:space="preserve">   Raspberry 4-Pack</t>
         </is>
       </c>
       <c r="C9" s="39">
@@ -1276,7 +1276,7 @@
     <row r="10">
       <c r="B10" s="34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Passionfruit 4-Pack</t>
+          <t xml:space="preserve">   Passion Fruit Pineapple 4-Pack</t>
         </is>
       </c>
       <c r="C10" s="39">
@@ -1386,7 +1386,7 @@
     <row r="16">
       <c r="B16" s="34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Pineapple Singles</t>
+          <t xml:space="preserve">   Raspberry Singles</t>
         </is>
       </c>
       <c r="C16" s="37">
@@ -1425,7 +1425,7 @@
     <row r="17">
       <c r="B17" s="34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Passionfruit Singles</t>
+          <t xml:space="preserve">   Passion Fruit Pineapple Singles</t>
         </is>
       </c>
       <c r="C17" s="37">
@@ -1503,7 +1503,7 @@
     <row r="19">
       <c r="B19" s="34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Pineapple 4-Pack</t>
+          <t xml:space="preserve">   Raspberry 4-Pack</t>
         </is>
       </c>
       <c r="C19" s="37">
@@ -1542,7 +1542,7 @@
     <row r="20">
       <c r="B20" s="34" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Passionfruit 4-Pack</t>
+          <t xml:space="preserve">   Passion Fruit Pineapple 4-Pack</t>
         </is>
       </c>
       <c r="C20" s="37">
@@ -1688,12 +1688,12 @@
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>Pineapple</t>
+          <t>Raspberry</t>
         </is>
       </c>
       <c r="D6" s="18" t="inlineStr">
         <is>
-          <t>Passionfruit</t>
+          <t>Passion Fruit Pineapple</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
@@ -1703,12 +1703,12 @@
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>Pineapple</t>
+          <t>Raspberry</t>
         </is>
       </c>
       <c r="G6" s="18" t="inlineStr">
         <is>
-          <t>Passionfruit</t>
+          <t>Passion Fruit Pineapple</t>
         </is>
       </c>
       <c r="H6" s="18" t="inlineStr">
@@ -3367,7 +3367,7 @@
       </c>
       <c r="D17" s="58" t="inlineStr">
         <is>
-          <t>Set to Pineapple, Passionfruit, Lime Lemon (editable on Assumptions).</t>
+          <t>Set to Raspberry, Passion Fruit Pineapple, Lime Lemon (editable on Assumptions).</t>
         </is>
       </c>
       <c r="E17" s="53" t="inlineStr">
@@ -3553,7 +3553,7 @@
       </c>
       <c r="C10" s="21" t="inlineStr">
         <is>
-          <t>3 flavours (Pineapple, Passionfruit, Lime Lemon) × Singles (12-ct) + 4-Pack = 6 SKUs; one fiscal year.</t>
+          <t>3 flavours (Raspberry, Passion Fruit Pineapple, Lime Lemon) × Singles (12-ct) + 4-Pack = 6 SKUs; one fiscal year.</t>
         </is>
       </c>
     </row>
@@ -3876,12 +3876,12 @@
       </c>
       <c r="C5" s="18" t="inlineStr">
         <is>
-          <t>Pineapple</t>
+          <t>Raspberry</t>
         </is>
       </c>
       <c r="D5" s="18" t="inlineStr">
         <is>
-          <t>Passionfruit</t>
+          <t>Passion Fruit Pineapple</t>
         </is>
       </c>
       <c r="E5" s="18" t="inlineStr">
@@ -3891,12 +3891,12 @@
       </c>
       <c r="F5" s="18" t="inlineStr">
         <is>
-          <t>Pineapple</t>
+          <t>Raspberry</t>
         </is>
       </c>
       <c r="G5" s="18" t="inlineStr">
         <is>
-          <t>Passionfruit</t>
+          <t>Passion Fruit Pineapple</t>
         </is>
       </c>
       <c r="H5" s="18" t="inlineStr">
@@ -3964,12 +3964,12 @@
       </c>
       <c r="C8" s="22" t="inlineStr">
         <is>
-          <t>Pineapple</t>
+          <t>Raspberry</t>
         </is>
       </c>
       <c r="D8" s="22" t="inlineStr">
         <is>
-          <t>Passionfruit</t>
+          <t>Passion Fruit Pineapple</t>
         </is>
       </c>
       <c r="E8" s="22" t="inlineStr">
@@ -3979,12 +3979,12 @@
       </c>
       <c r="F8" s="22" t="inlineStr">
         <is>
-          <t>Pineapple</t>
+          <t>Raspberry</t>
         </is>
       </c>
       <c r="G8" s="22" t="inlineStr">
         <is>
-          <t>Passionfruit</t>
+          <t>Passion Fruit Pineapple</t>
         </is>
       </c>
       <c r="H8" s="22" t="inlineStr">
@@ -5370,12 +5370,12 @@
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>Pineapple</t>
+          <t>Raspberry</t>
         </is>
       </c>
       <c r="D6" s="18" t="inlineStr">
         <is>
-          <t>Passionfruit</t>
+          <t>Passion Fruit Pineapple</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
@@ -5385,12 +5385,12 @@
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>Pineapple</t>
+          <t>Raspberry</t>
         </is>
       </c>
       <c r="G6" s="18" t="inlineStr">
         <is>
-          <t>Passionfruit</t>
+          <t>Passion Fruit Pineapple</t>
         </is>
       </c>
       <c r="H6" s="18" t="inlineStr">
@@ -6391,12 +6391,12 @@
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>Pineapple</t>
+          <t>Raspberry</t>
         </is>
       </c>
       <c r="D6" s="18" t="inlineStr">
         <is>
-          <t>Passionfruit</t>
+          <t>Passion Fruit Pineapple</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
@@ -6406,12 +6406,12 @@
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>Pineapple</t>
+          <t>Raspberry</t>
         </is>
       </c>
       <c r="G6" s="18" t="inlineStr">
         <is>
-          <t>Passionfruit</t>
+          <t>Passion Fruit Pineapple</t>
         </is>
       </c>
       <c r="H6" s="18" t="inlineStr">
@@ -7412,12 +7412,12 @@
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>Pineapple</t>
+          <t>Raspberry</t>
         </is>
       </c>
       <c r="D6" s="18" t="inlineStr">
         <is>
-          <t>Passionfruit</t>
+          <t>Passion Fruit Pineapple</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
@@ -7427,12 +7427,12 @@
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>Pineapple</t>
+          <t>Raspberry</t>
         </is>
       </c>
       <c r="G6" s="18" t="inlineStr">
         <is>
-          <t>Passionfruit</t>
+          <t>Passion Fruit Pineapple</t>
         </is>
       </c>
       <c r="H6" s="18" t="inlineStr">
@@ -8433,12 +8433,12 @@
       </c>
       <c r="C6" s="18" t="inlineStr">
         <is>
-          <t>Pineapple</t>
+          <t>Raspberry</t>
         </is>
       </c>
       <c r="D6" s="18" t="inlineStr">
         <is>
-          <t>Passionfruit</t>
+          <t>Passion Fruit Pineapple</t>
         </is>
       </c>
       <c r="E6" s="18" t="inlineStr">
@@ -8448,12 +8448,12 @@
       </c>
       <c r="F6" s="18" t="inlineStr">
         <is>
-          <t>Pineapple</t>
+          <t>Raspberry</t>
         </is>
       </c>
       <c r="G6" s="18" t="inlineStr">
         <is>
-          <t>Passionfruit</t>
+          <t>Passion Fruit Pineapple</t>
         </is>
       </c>
       <c r="H6" s="18" t="inlineStr">

</xml_diff>